<commit_message>
Estadisticos Primer Parcial 20231 SD2
</commit_message>
<xml_diff>
--- a/DetalleXDocente20231.xlsx
+++ b/DetalleXDocente20231.xlsx
@@ -965,7 +965,7 @@
         <v>99</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E6">
         <v>12</v>
@@ -974,7 +974,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="H6" s="1">
         <v>0</v>
@@ -983,10 +983,10 @@
         <v>8.199999999999999</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K6" s="1">
-        <v>14.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -997,7 +997,7 @@
         <v>100</v>
       </c>
       <c r="D7">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E7">
         <v>92</v>
@@ -1006,19 +1006,19 @@
         <v>8</v>
       </c>
       <c r="G7" s="1">
-        <v>90.2</v>
+        <v>92</v>
       </c>
       <c r="H7" s="1">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="I7" s="2">
         <v>8.1</v>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1618,7 +1618,7 @@
         <v>99</v>
       </c>
       <c r="D25">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E25">
         <v>12</v>
@@ -1627,7 +1627,7 @@
         <v>0</v>
       </c>
       <c r="G25" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="H25" s="1">
         <v>0</v>
@@ -1636,10 +1636,10 @@
         <v>9.1</v>
       </c>
       <c r="J25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K25" s="1">
-        <v>14.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -1650,7 +1650,7 @@
         <v>100</v>
       </c>
       <c r="D26">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E26">
         <v>12</v>
@@ -1659,7 +1659,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="H26" s="1">
         <v>0</v>
@@ -1668,10 +1668,10 @@
         <v>9.1</v>
       </c>
       <c r="J26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K26" s="1">
-        <v>14.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -1790,7 +1790,7 @@
         <v>110</v>
       </c>
       <c r="D30">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E30">
         <v>31</v>
@@ -1799,7 +1799,7 @@
         <v>0</v>
       </c>
       <c r="G30" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H30" s="1">
         <v>0</v>
@@ -1808,10 +1808,10 @@
         <v>9.4</v>
       </c>
       <c r="J30">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K30" s="1">
-        <v>6.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -1822,7 +1822,7 @@
         <v>100</v>
       </c>
       <c r="D31">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E31">
         <v>126</v>
@@ -1831,19 +1831,19 @@
         <v>4</v>
       </c>
       <c r="G31" s="1">
-        <v>95.5</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H31" s="1">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="I31" s="2">
         <v>9</v>
       </c>
       <c r="J31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K31" s="1">
-        <v>1.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -2443,7 +2443,7 @@
         <v>99</v>
       </c>
       <c r="D49">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E49">
         <v>6</v>
@@ -2452,19 +2452,19 @@
         <v>6</v>
       </c>
       <c r="G49" s="1">
-        <v>42.9</v>
+        <v>50</v>
       </c>
       <c r="H49" s="1">
-        <v>42.9</v>
+        <v>50</v>
       </c>
       <c r="I49" s="2">
         <v>6.3</v>
       </c>
       <c r="J49">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K49" s="1">
-        <v>14.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -2475,7 +2475,7 @@
         <v>100</v>
       </c>
       <c r="D50">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E50">
         <v>72</v>
@@ -2484,19 +2484,19 @@
         <v>52</v>
       </c>
       <c r="G50" s="1">
-        <v>57.1</v>
+        <v>58.1</v>
       </c>
       <c r="H50" s="1">
-        <v>41.3</v>
+        <v>41.9</v>
       </c>
       <c r="I50" s="2">
         <v>6.4</v>
       </c>
       <c r="J50">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K50" s="1">
-        <v>1.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -3341,7 +3341,7 @@
         <v>110</v>
       </c>
       <c r="D75">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E75">
         <v>31</v>
@@ -3350,7 +3350,7 @@
         <v>0</v>
       </c>
       <c r="G75" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H75" s="1">
         <v>0</v>
@@ -3359,10 +3359,10 @@
         <v>9.6</v>
       </c>
       <c r="J75">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K75" s="1">
-        <v>6.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:11">
@@ -3478,7 +3478,7 @@
         <v>100</v>
       </c>
       <c r="D79">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E79">
         <v>230</v>
@@ -3487,19 +3487,19 @@
         <v>9</v>
       </c>
       <c r="G79" s="1">
-        <v>95.40000000000001</v>
+        <v>96.2</v>
       </c>
       <c r="H79" s="1">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="I79" s="2">
         <v>8.800000000000001</v>
       </c>
       <c r="J79">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K79" s="1">
-        <v>0.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80" spans="1:11">
@@ -4320,7 +4320,7 @@
         <v>110</v>
       </c>
       <c r="D104">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E104">
         <v>0</v>
@@ -4335,7 +4335,7 @@
         <v>0</v>
       </c>
       <c r="J104">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K104" s="1">
         <v>100</v>
@@ -4413,7 +4413,7 @@
         <v>100</v>
       </c>
       <c r="D107">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E107">
         <v>0</v>
@@ -4428,7 +4428,7 @@
         <v>0</v>
       </c>
       <c r="J107">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="K107" s="1">
         <v>100</v>
@@ -5034,7 +5034,7 @@
         <v>99</v>
       </c>
       <c r="D125">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E125">
         <v>8</v>
@@ -5043,19 +5043,19 @@
         <v>4</v>
       </c>
       <c r="G125" s="1">
-        <v>57.1</v>
+        <v>66.7</v>
       </c>
       <c r="H125" s="1">
-        <v>28.6</v>
+        <v>33.3</v>
       </c>
       <c r="I125" s="2">
         <v>7.3</v>
       </c>
       <c r="J125">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K125" s="1">
-        <v>14.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126" spans="1:11">
@@ -5066,7 +5066,7 @@
         <v>100</v>
       </c>
       <c r="D126">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E126">
         <v>161</v>
@@ -5075,19 +5075,19 @@
         <v>27</v>
       </c>
       <c r="G126" s="1">
-        <v>84.7</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="H126" s="1">
-        <v>14.2</v>
+        <v>14.4</v>
       </c>
       <c r="I126" s="2">
         <v>8.1</v>
       </c>
       <c r="J126">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K126" s="1">
-        <v>1.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127" spans="1:11">
@@ -5652,7 +5652,7 @@
         <v>110</v>
       </c>
       <c r="D143">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E143">
         <v>28</v>
@@ -5661,19 +5661,19 @@
         <v>3</v>
       </c>
       <c r="G143" s="1">
-        <v>84.8</v>
+        <v>90.3</v>
       </c>
       <c r="H143" s="1">
-        <v>9.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I143" s="2">
         <v>7.4</v>
       </c>
       <c r="J143">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K143" s="1">
-        <v>6.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:11">
@@ -5719,7 +5719,7 @@
         <v>100</v>
       </c>
       <c r="D145">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E145">
         <v>107</v>
@@ -5728,19 +5728,19 @@
         <v>3</v>
       </c>
       <c r="G145" s="1">
-        <v>83.59999999999999</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="H145" s="1">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="I145" s="2">
         <v>7.4</v>
       </c>
       <c r="J145">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K145" s="1">
-        <v>2.3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="146" spans="1:11">
@@ -5824,7 +5824,7 @@
         <v>110</v>
       </c>
       <c r="D148">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E148">
         <v>31</v>
@@ -5833,7 +5833,7 @@
         <v>0</v>
       </c>
       <c r="G148" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H148" s="1">
         <v>0</v>
@@ -5842,10 +5842,10 @@
         <v>9.199999999999999</v>
       </c>
       <c r="J148">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K148" s="1">
-        <v>6.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149" spans="1:11">
@@ -5856,7 +5856,7 @@
         <v>100</v>
       </c>
       <c r="D149">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E149">
         <v>98</v>
@@ -5865,7 +5865,7 @@
         <v>3</v>
       </c>
       <c r="G149" s="1">
-        <v>94.2</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="H149" s="1">
         <v>2.9</v>
@@ -5874,10 +5874,10 @@
         <v>8.4</v>
       </c>
       <c r="J149">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K149" s="1">
-        <v>2.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150" spans="1:11">
@@ -6894,7 +6894,7 @@
         <v>110</v>
       </c>
       <c r="D179">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E179">
         <v>31</v>
@@ -6903,7 +6903,7 @@
         <v>0</v>
       </c>
       <c r="G179" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H179" s="1">
         <v>0</v>
@@ -6912,10 +6912,10 @@
         <v>9.199999999999999</v>
       </c>
       <c r="J179">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K179" s="1">
-        <v>6.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="180" spans="1:11">
@@ -6926,7 +6926,7 @@
         <v>100</v>
       </c>
       <c r="D180">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E180">
         <v>209</v>
@@ -6935,19 +6935,19 @@
         <v>28</v>
       </c>
       <c r="G180" s="1">
-        <v>87.09999999999999</v>
+        <v>87.8</v>
       </c>
       <c r="H180" s="1">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="I180" s="2">
         <v>7.5</v>
       </c>
       <c r="J180">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K180" s="1">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="181" spans="1:11">
@@ -7101,7 +7101,7 @@
         <v>99</v>
       </c>
       <c r="D185">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E185">
         <v>12</v>
@@ -7110,7 +7110,7 @@
         <v>0</v>
       </c>
       <c r="G185" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="H185" s="1">
         <v>0</v>
@@ -7119,10 +7119,10 @@
         <v>7.6</v>
       </c>
       <c r="J185">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K185" s="1">
-        <v>14.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="186" spans="1:11">
@@ -7133,7 +7133,7 @@
         <v>100</v>
       </c>
       <c r="D186">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E186">
         <v>132</v>
@@ -7142,7 +7142,7 @@
         <v>0</v>
       </c>
       <c r="G186" s="1">
-        <v>98.5</v>
+        <v>100</v>
       </c>
       <c r="H186" s="1">
         <v>0</v>
@@ -7151,10 +7151,10 @@
         <v>7.3</v>
       </c>
       <c r="J186">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K186" s="1">
-        <v>1.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="187" spans="1:11">
@@ -8631,7 +8631,7 @@
         <v>99</v>
       </c>
       <c r="D230">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E230">
         <v>2</v>
@@ -8640,19 +8640,19 @@
         <v>10</v>
       </c>
       <c r="G230" s="1">
-        <v>14.3</v>
+        <v>16.7</v>
       </c>
       <c r="H230" s="1">
-        <v>71.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="I230" s="2">
         <v>4.8</v>
       </c>
       <c r="J230">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K230" s="1">
-        <v>14.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="231" spans="1:11">
@@ -8663,7 +8663,7 @@
         <v>100</v>
       </c>
       <c r="D231">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E231">
         <v>2</v>
@@ -8672,19 +8672,19 @@
         <v>10</v>
       </c>
       <c r="G231" s="1">
-        <v>14.3</v>
+        <v>16.7</v>
       </c>
       <c r="H231" s="1">
-        <v>71.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="I231" s="2">
         <v>4.8</v>
       </c>
       <c r="J231">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K231" s="1">
-        <v>14.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="232" spans="1:11">
@@ -9930,7 +9930,7 @@
         <v>99</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -9942,10 +9942,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="J6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K6" s="1">
         <v>100</v>
@@ -9959,7 +9959,7 @@
         <v>100</v>
       </c>
       <c r="D7">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -9971,10 +9971,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="1">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J7">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="K7" s="1">
         <v>100</v>
@@ -10526,7 +10526,7 @@
         <v>99</v>
       </c>
       <c r="D25">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -10538,10 +10538,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="J25">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K25" s="1">
         <v>100</v>
@@ -10555,7 +10555,7 @@
         <v>100</v>
       </c>
       <c r="D26">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -10567,10 +10567,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="J26">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K26" s="1">
         <v>100</v>
@@ -10683,7 +10683,7 @@
         <v>110</v>
       </c>
       <c r="D30">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -10695,10 +10695,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="J30">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K30" s="1">
         <v>100</v>
@@ -10712,7 +10712,7 @@
         <v>100</v>
       </c>
       <c r="D31">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -10724,10 +10724,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="1">
-        <v>98.5</v>
+        <v>100</v>
       </c>
       <c r="J31">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K31" s="1">
         <v>100</v>
@@ -11279,7 +11279,7 @@
         <v>99</v>
       </c>
       <c r="D49">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -11291,10 +11291,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="J49">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K49" s="1">
         <v>100</v>
@@ -11308,7 +11308,7 @@
         <v>100</v>
       </c>
       <c r="D50">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E50">
         <v>0</v>
@@ -11320,10 +11320,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="1">
-        <v>98.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="J50">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K50" s="1">
         <v>100</v>
@@ -12099,7 +12099,7 @@
         <v>110</v>
       </c>
       <c r="D75">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E75">
         <v>0</v>
@@ -12111,10 +12111,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="J75">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K75" s="1">
         <v>100</v>
@@ -12224,7 +12224,7 @@
         <v>100</v>
       </c>
       <c r="D79">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E79">
         <v>0</v>
@@ -12236,10 +12236,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="1">
-        <v>99.2</v>
+        <v>100</v>
       </c>
       <c r="J79">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="K79" s="1">
         <v>100</v>
@@ -13015,7 +13015,7 @@
         <v>110</v>
       </c>
       <c r="D104">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E104">
         <v>0</v>
@@ -13030,7 +13030,7 @@
         <v>0</v>
       </c>
       <c r="J104">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K104" s="1">
         <v>100</v>
@@ -13108,7 +13108,7 @@
         <v>100</v>
       </c>
       <c r="D107">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E107">
         <v>0</v>
@@ -13123,7 +13123,7 @@
         <v>0</v>
       </c>
       <c r="J107">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="K107" s="1">
         <v>100</v>
@@ -13678,7 +13678,7 @@
         <v>99</v>
       </c>
       <c r="D125">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E125">
         <v>0</v>
@@ -13690,10 +13690,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="J125">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K125" s="1">
         <v>100</v>
@@ -13707,7 +13707,7 @@
         <v>100</v>
       </c>
       <c r="D126">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E126">
         <v>0</v>
@@ -13719,10 +13719,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="1">
-        <v>98.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="J126">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="K126" s="1">
         <v>100</v>
@@ -14242,7 +14242,7 @@
         <v>110</v>
       </c>
       <c r="D143">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E143">
         <v>0</v>
@@ -14254,10 +14254,10 @@
         <v>0</v>
       </c>
       <c r="H143" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="J143">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K143" s="1">
         <v>100</v>
@@ -14303,7 +14303,7 @@
         <v>100</v>
       </c>
       <c r="D145">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E145">
         <v>0</v>
@@ -14315,10 +14315,10 @@
         <v>0</v>
       </c>
       <c r="H145" s="1">
-        <v>85.90000000000001</v>
+        <v>87.3</v>
       </c>
       <c r="J145">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K145" s="1">
         <v>100</v>
@@ -14399,7 +14399,7 @@
         <v>110</v>
       </c>
       <c r="D148">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E148">
         <v>0</v>
@@ -14411,10 +14411,10 @@
         <v>0</v>
       </c>
       <c r="H148" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="J148">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K148" s="1">
         <v>100</v>
@@ -14428,7 +14428,7 @@
         <v>100</v>
       </c>
       <c r="D149">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E149">
         <v>0</v>
@@ -14440,10 +14440,10 @@
         <v>0</v>
       </c>
       <c r="H149" s="1">
-        <v>97.09999999999999</v>
+        <v>99</v>
       </c>
       <c r="J149">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="K149" s="1">
         <v>100</v>
@@ -15376,7 +15376,7 @@
         <v>110</v>
       </c>
       <c r="D179">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E179">
         <v>0</v>
@@ -15388,10 +15388,10 @@
         <v>0</v>
       </c>
       <c r="H179" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="J179">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K179" s="1">
         <v>100</v>
@@ -15405,7 +15405,7 @@
         <v>100</v>
       </c>
       <c r="D180">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E180">
         <v>0</v>
@@ -15417,10 +15417,10 @@
         <v>0</v>
       </c>
       <c r="H180" s="1">
-        <v>98.8</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="J180">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="K180" s="1">
         <v>100</v>
@@ -15565,7 +15565,7 @@
         <v>99</v>
       </c>
       <c r="D185">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E185">
         <v>0</v>
@@ -15577,10 +15577,10 @@
         <v>0</v>
       </c>
       <c r="H185" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="J185">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K185" s="1">
         <v>100</v>
@@ -15594,7 +15594,7 @@
         <v>100</v>
       </c>
       <c r="D186">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E186">
         <v>0</v>
@@ -15606,10 +15606,10 @@
         <v>0</v>
       </c>
       <c r="H186" s="1">
-        <v>98.5</v>
+        <v>100</v>
       </c>
       <c r="J186">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K186" s="1">
         <v>100</v>
@@ -16969,7 +16969,7 @@
         <v>99</v>
       </c>
       <c r="D230">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E230">
         <v>0</v>
@@ -16981,10 +16981,10 @@
         <v>0</v>
       </c>
       <c r="H230" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="J230">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K230" s="1">
         <v>100</v>
@@ -16998,7 +16998,7 @@
         <v>100</v>
       </c>
       <c r="D231">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E231">
         <v>0</v>
@@ -17010,10 +17010,10 @@
         <v>0</v>
       </c>
       <c r="H231" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="J231">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K231" s="1">
         <v>100</v>
@@ -18199,7 +18199,7 @@
         <v>99</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E6">
         <v>12</v>
@@ -18208,7 +18208,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="H6" s="1">
         <v>0</v>
@@ -18217,7 +18217,7 @@
         <v>8.199999999999999</v>
       </c>
       <c r="J6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K6" s="1">
         <v>100</v>
@@ -18231,7 +18231,7 @@
         <v>100</v>
       </c>
       <c r="D7">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E7">
         <v>92</v>
@@ -18240,16 +18240,16 @@
         <v>8</v>
       </c>
       <c r="G7" s="1">
-        <v>90.2</v>
+        <v>92</v>
       </c>
       <c r="H7" s="1">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="I7" s="2">
         <v>8.1</v>
       </c>
       <c r="J7">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="K7" s="1">
         <v>100</v>
@@ -18852,7 +18852,7 @@
         <v>99</v>
       </c>
       <c r="D25">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E25">
         <v>12</v>
@@ -18861,7 +18861,7 @@
         <v>0</v>
       </c>
       <c r="G25" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="H25" s="1">
         <v>0</v>
@@ -18870,7 +18870,7 @@
         <v>9.1</v>
       </c>
       <c r="J25">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K25" s="1">
         <v>100</v>
@@ -18884,7 +18884,7 @@
         <v>100</v>
       </c>
       <c r="D26">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E26">
         <v>12</v>
@@ -18893,7 +18893,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="H26" s="1">
         <v>0</v>
@@ -18902,7 +18902,7 @@
         <v>9.1</v>
       </c>
       <c r="J26">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K26" s="1">
         <v>100</v>
@@ -19024,7 +19024,7 @@
         <v>110</v>
       </c>
       <c r="D30">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E30">
         <v>31</v>
@@ -19033,7 +19033,7 @@
         <v>0</v>
       </c>
       <c r="G30" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H30" s="1">
         <v>0</v>
@@ -19042,7 +19042,7 @@
         <v>9.4</v>
       </c>
       <c r="J30">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K30" s="1">
         <v>100</v>
@@ -19056,7 +19056,7 @@
         <v>100</v>
       </c>
       <c r="D31">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E31">
         <v>126</v>
@@ -19065,16 +19065,16 @@
         <v>4</v>
       </c>
       <c r="G31" s="1">
-        <v>95.5</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H31" s="1">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="I31" s="2">
         <v>9</v>
       </c>
       <c r="J31">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K31" s="1">
         <v>100</v>
@@ -19677,7 +19677,7 @@
         <v>99</v>
       </c>
       <c r="D49">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E49">
         <v>6</v>
@@ -19686,16 +19686,16 @@
         <v>6</v>
       </c>
       <c r="G49" s="1">
-        <v>42.9</v>
+        <v>50</v>
       </c>
       <c r="H49" s="1">
-        <v>42.9</v>
+        <v>50</v>
       </c>
       <c r="I49" s="2">
         <v>6.3</v>
       </c>
       <c r="J49">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K49" s="1">
         <v>100</v>
@@ -19709,7 +19709,7 @@
         <v>100</v>
       </c>
       <c r="D50">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E50">
         <v>72</v>
@@ -19718,16 +19718,16 @@
         <v>52</v>
       </c>
       <c r="G50" s="1">
-        <v>57.1</v>
+        <v>58.1</v>
       </c>
       <c r="H50" s="1">
-        <v>41.3</v>
+        <v>41.9</v>
       </c>
       <c r="I50" s="2">
         <v>6.4</v>
       </c>
       <c r="J50">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K50" s="1">
         <v>100</v>
@@ -20575,7 +20575,7 @@
         <v>110</v>
       </c>
       <c r="D75">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E75">
         <v>31</v>
@@ -20584,7 +20584,7 @@
         <v>0</v>
       </c>
       <c r="G75" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H75" s="1">
         <v>0</v>
@@ -20593,7 +20593,7 @@
         <v>9.6</v>
       </c>
       <c r="J75">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K75" s="1">
         <v>100</v>
@@ -20712,7 +20712,7 @@
         <v>100</v>
       </c>
       <c r="D79">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E79">
         <v>230</v>
@@ -20721,16 +20721,16 @@
         <v>9</v>
       </c>
       <c r="G79" s="1">
-        <v>95.40000000000001</v>
+        <v>96.2</v>
       </c>
       <c r="H79" s="1">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="I79" s="2">
         <v>8.800000000000001</v>
       </c>
       <c r="J79">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="K79" s="1">
         <v>100</v>
@@ -21554,7 +21554,7 @@
         <v>110</v>
       </c>
       <c r="D104">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E104">
         <v>0</v>
@@ -21569,7 +21569,7 @@
         <v>0</v>
       </c>
       <c r="J104">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K104" s="1">
         <v>100</v>
@@ -21647,7 +21647,7 @@
         <v>100</v>
       </c>
       <c r="D107">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E107">
         <v>0</v>
@@ -21662,7 +21662,7 @@
         <v>0</v>
       </c>
       <c r="J107">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="K107" s="1">
         <v>100</v>
@@ -22268,7 +22268,7 @@
         <v>99</v>
       </c>
       <c r="D125">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E125">
         <v>8</v>
@@ -22277,16 +22277,16 @@
         <v>4</v>
       </c>
       <c r="G125" s="1">
-        <v>57.1</v>
+        <v>66.7</v>
       </c>
       <c r="H125" s="1">
-        <v>28.6</v>
+        <v>33.3</v>
       </c>
       <c r="I125" s="2">
         <v>7.3</v>
       </c>
       <c r="J125">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K125" s="1">
         <v>100</v>
@@ -22300,7 +22300,7 @@
         <v>100</v>
       </c>
       <c r="D126">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E126">
         <v>161</v>
@@ -22309,16 +22309,16 @@
         <v>27</v>
       </c>
       <c r="G126" s="1">
-        <v>84.7</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="H126" s="1">
-        <v>14.2</v>
+        <v>14.4</v>
       </c>
       <c r="I126" s="2">
         <v>8.1</v>
       </c>
       <c r="J126">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="K126" s="1">
         <v>100</v>
@@ -22886,7 +22886,7 @@
         <v>110</v>
       </c>
       <c r="D143">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E143">
         <v>28</v>
@@ -22895,16 +22895,16 @@
         <v>3</v>
       </c>
       <c r="G143" s="1">
-        <v>84.8</v>
+        <v>90.3</v>
       </c>
       <c r="H143" s="1">
-        <v>9.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I143" s="2">
         <v>7.4</v>
       </c>
       <c r="J143">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K143" s="1">
         <v>100</v>
@@ -22953,7 +22953,7 @@
         <v>100</v>
       </c>
       <c r="D145">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E145">
         <v>107</v>
@@ -22962,16 +22962,16 @@
         <v>18</v>
       </c>
       <c r="G145" s="1">
-        <v>83.59999999999999</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="H145" s="1">
-        <v>14.1</v>
+        <v>14.3</v>
       </c>
       <c r="I145" s="2">
         <v>7.1</v>
       </c>
       <c r="J145">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K145" s="1">
         <v>100</v>
@@ -23058,7 +23058,7 @@
         <v>110</v>
       </c>
       <c r="D148">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E148">
         <v>31</v>
@@ -23067,7 +23067,7 @@
         <v>0</v>
       </c>
       <c r="G148" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H148" s="1">
         <v>0</v>
@@ -23076,7 +23076,7 @@
         <v>9.199999999999999</v>
       </c>
       <c r="J148">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K148" s="1">
         <v>100</v>
@@ -23090,7 +23090,7 @@
         <v>100</v>
       </c>
       <c r="D149">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E149">
         <v>98</v>
@@ -23099,7 +23099,7 @@
         <v>3</v>
       </c>
       <c r="G149" s="1">
-        <v>94.2</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="H149" s="1">
         <v>2.9</v>
@@ -23108,7 +23108,7 @@
         <v>8.4</v>
       </c>
       <c r="J149">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="K149" s="1">
         <v>100</v>
@@ -24128,7 +24128,7 @@
         <v>110</v>
       </c>
       <c r="D179">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E179">
         <v>31</v>
@@ -24137,7 +24137,7 @@
         <v>0</v>
       </c>
       <c r="G179" s="1">
-        <v>93.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H179" s="1">
         <v>0</v>
@@ -24146,7 +24146,7 @@
         <v>9.199999999999999</v>
       </c>
       <c r="J179">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K179" s="1">
         <v>100</v>
@@ -24160,7 +24160,7 @@
         <v>100</v>
       </c>
       <c r="D180">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E180">
         <v>209</v>
@@ -24169,16 +24169,16 @@
         <v>28</v>
       </c>
       <c r="G180" s="1">
-        <v>87.09999999999999</v>
+        <v>87.8</v>
       </c>
       <c r="H180" s="1">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="I180" s="2">
         <v>7.5</v>
       </c>
       <c r="J180">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="K180" s="1">
         <v>100</v>
@@ -24335,7 +24335,7 @@
         <v>99</v>
       </c>
       <c r="D185">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E185">
         <v>12</v>
@@ -24344,7 +24344,7 @@
         <v>0</v>
       </c>
       <c r="G185" s="1">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="H185" s="1">
         <v>0</v>
@@ -24353,7 +24353,7 @@
         <v>7.6</v>
       </c>
       <c r="J185">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K185" s="1">
         <v>100</v>
@@ -24367,7 +24367,7 @@
         <v>100</v>
       </c>
       <c r="D186">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E186">
         <v>132</v>
@@ -24376,7 +24376,7 @@
         <v>0</v>
       </c>
       <c r="G186" s="1">
-        <v>98.5</v>
+        <v>100</v>
       </c>
       <c r="H186" s="1">
         <v>0</v>
@@ -24385,7 +24385,7 @@
         <v>7.3</v>
       </c>
       <c r="J186">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K186" s="1">
         <v>100</v>
@@ -25865,7 +25865,7 @@
         <v>99</v>
       </c>
       <c r="D230">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E230">
         <v>2</v>
@@ -25874,16 +25874,16 @@
         <v>10</v>
       </c>
       <c r="G230" s="1">
-        <v>14.3</v>
+        <v>16.7</v>
       </c>
       <c r="H230" s="1">
-        <v>71.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="I230" s="2">
         <v>5.3</v>
       </c>
       <c r="J230">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K230" s="1">
         <v>100</v>
@@ -25897,7 +25897,7 @@
         <v>100</v>
       </c>
       <c r="D231">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E231">
         <v>2</v>
@@ -25906,16 +25906,16 @@
         <v>10</v>
       </c>
       <c r="G231" s="1">
-        <v>14.3</v>
+        <v>16.7</v>
       </c>
       <c r="H231" s="1">
-        <v>71.40000000000001</v>
+        <v>83.3</v>
       </c>
       <c r="I231" s="2">
         <v>5.3</v>
       </c>
       <c r="J231">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K231" s="1">
         <v>100</v>

</xml_diff>

<commit_message>
Estadisticos Segundo Parcial 20231 3N
</commit_message>
<xml_diff>
--- a/DetalleXDocente20231.xlsx
+++ b/DetalleXDocente20231.xlsx
@@ -5003,13 +5003,13 @@
         <v>36</v>
       </c>
       <c r="E123">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F123">
         <v>2</v>
       </c>
       <c r="G123" s="1">
-        <v>91.7</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="H123" s="1">
         <v>5.6</v>
@@ -5018,10 +5018,10 @@
         <v>8.6</v>
       </c>
       <c r="J123">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K123" s="1">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124" spans="1:11">
@@ -5105,13 +5105,13 @@
         <v>189</v>
       </c>
       <c r="E126">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F126">
         <v>27</v>
       </c>
       <c r="G126" s="1">
-        <v>85.2</v>
+        <v>85.7</v>
       </c>
       <c r="H126" s="1">
         <v>14.3</v>
@@ -5120,10 +5120,10 @@
         <v>8.1</v>
       </c>
       <c r="J126">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K126" s="1">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127" spans="1:11">
@@ -7761,22 +7761,22 @@
         <v>14</v>
       </c>
       <c r="F203">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G203" s="1">
         <v>73.7</v>
       </c>
       <c r="H203" s="1">
-        <v>21.1</v>
+        <v>26.3</v>
       </c>
       <c r="I203" s="2">
         <v>6.4</v>
       </c>
       <c r="J203">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K203" s="1">
-        <v>5.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="204" spans="1:11">
@@ -7793,22 +7793,22 @@
         <v>84</v>
       </c>
       <c r="F204">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G204" s="1">
         <v>63.2</v>
       </c>
       <c r="H204" s="1">
-        <v>36.1</v>
+        <v>36.8</v>
       </c>
       <c r="I204" s="2">
         <v>5.9</v>
       </c>
       <c r="J204">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K204" s="1">
-        <v>0.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205" spans="1:11">
@@ -9268,22 +9268,22 @@
         <v>14</v>
       </c>
       <c r="F247">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G247" s="1">
         <v>73.7</v>
       </c>
       <c r="H247" s="1">
-        <v>21.1</v>
+        <v>26.3</v>
       </c>
       <c r="I247" s="2">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
       <c r="J247">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K247" s="1">
-        <v>5.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248" spans="1:11">
@@ -9370,22 +9370,22 @@
         <v>118</v>
       </c>
       <c r="F250">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G250" s="1">
         <v>62.8</v>
       </c>
       <c r="H250" s="1">
-        <v>36.2</v>
+        <v>36.7</v>
       </c>
       <c r="I250" s="2">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="J250">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K250" s="1">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="251" spans="1:11">
@@ -10387,22 +10387,25 @@
         <v>38</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F17">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="G17" s="1">
-        <v>0</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="H17" s="1">
-        <v>100</v>
+        <v>18.4</v>
+      </c>
+      <c r="I17" s="2">
+        <v>7.8</v>
       </c>
       <c r="J17">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="K17" s="1">
-        <v>100</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -10419,22 +10422,25 @@
         <v>38</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F18">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="G18" s="1">
-        <v>0</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="H18" s="1">
-        <v>100</v>
+        <v>18.4</v>
+      </c>
+      <c r="I18" s="2">
+        <v>7.1</v>
       </c>
       <c r="J18">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="K18" s="1">
-        <v>100</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -10448,25 +10454,25 @@
         <v>160</v>
       </c>
       <c r="E19">
-        <v>79</v>
+        <v>141</v>
       </c>
       <c r="F19">
-        <v>81</v>
+        <v>19</v>
       </c>
       <c r="G19" s="1">
-        <v>49.4</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="H19" s="1">
-        <v>50.6</v>
+        <v>11.9</v>
       </c>
       <c r="I19" s="2">
-        <v>8.300000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="J19">
-        <v>76</v>
+        <v>2</v>
       </c>
       <c r="K19" s="1">
-        <v>47.5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -10929,22 +10935,25 @@
         <v>39</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F33">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="G33" s="1">
-        <v>0</v>
+        <v>56.4</v>
       </c>
       <c r="H33" s="1">
-        <v>100</v>
+        <v>43.6</v>
+      </c>
+      <c r="I33" s="2">
+        <v>6.7</v>
       </c>
       <c r="J33">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K33" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -10961,22 +10970,25 @@
         <v>39</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F34">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="G34" s="1">
-        <v>0</v>
+        <v>61.5</v>
       </c>
       <c r="H34" s="1">
-        <v>100</v>
+        <v>38.5</v>
+      </c>
+      <c r="I34" s="2">
+        <v>6.3</v>
       </c>
       <c r="J34">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K34" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -10993,22 +11005,25 @@
         <v>37</v>
       </c>
       <c r="E35">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F35">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="G35" s="1">
-        <v>0</v>
+        <v>40.5</v>
       </c>
       <c r="H35" s="1">
-        <v>100</v>
+        <v>59.5</v>
+      </c>
+      <c r="I35" s="2">
+        <v>6.2</v>
       </c>
       <c r="J35">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K35" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -11057,25 +11072,25 @@
         <v>170</v>
       </c>
       <c r="E37">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="F37">
-        <v>145</v>
+        <v>84</v>
       </c>
       <c r="G37" s="1">
-        <v>14.7</v>
+        <v>50.6</v>
       </c>
       <c r="H37" s="1">
-        <v>85.3</v>
+        <v>49.4</v>
       </c>
       <c r="I37" s="2">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="J37">
-        <v>115</v>
+        <v>0</v>
       </c>
       <c r="K37" s="1">
-        <v>67.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -13261,22 +13276,25 @@
         <v>30</v>
       </c>
       <c r="E101">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F101">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G101" s="1">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="H101" s="1">
-        <v>100</v>
+        <v>33.3</v>
+      </c>
+      <c r="I101" s="2">
+        <v>6.3</v>
       </c>
       <c r="J101">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K101" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102" spans="1:11">
@@ -13293,22 +13311,25 @@
         <v>38</v>
       </c>
       <c r="E102">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F102">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="G102" s="1">
-        <v>0</v>
+        <v>94.7</v>
       </c>
       <c r="H102" s="1">
-        <v>100</v>
+        <v>5.3</v>
+      </c>
+      <c r="I102" s="2">
+        <v>8.1</v>
       </c>
       <c r="J102">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="K102" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103" spans="1:11">
@@ -13325,22 +13346,25 @@
         <v>25</v>
       </c>
       <c r="E103">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F103">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="G103" s="1">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H103" s="1">
-        <v>100</v>
+        <v>20</v>
+      </c>
+      <c r="I103" s="2">
+        <v>7.3</v>
       </c>
       <c r="J103">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K103" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104" spans="1:11">
@@ -13357,22 +13381,25 @@
         <v>31</v>
       </c>
       <c r="E104">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F104">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="G104" s="1">
-        <v>0</v>
+        <v>90.3</v>
       </c>
       <c r="H104" s="1">
-        <v>100</v>
+        <v>9.699999999999999</v>
+      </c>
+      <c r="I104" s="2">
+        <v>8.199999999999999</v>
       </c>
       <c r="J104">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K104" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:11">
@@ -13389,22 +13416,25 @@
         <v>36</v>
       </c>
       <c r="E105">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F105">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="G105" s="1">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H105" s="1">
-        <v>100</v>
+        <v>25</v>
+      </c>
+      <c r="I105" s="2">
+        <v>7.6</v>
       </c>
       <c r="J105">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K105" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:11">
@@ -13421,22 +13451,25 @@
         <v>28</v>
       </c>
       <c r="E106">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F106">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="G106" s="1">
-        <v>0</v>
+        <v>89.3</v>
       </c>
       <c r="H106" s="1">
-        <v>100</v>
+        <v>10.7</v>
+      </c>
+      <c r="I106" s="2">
+        <v>6.5</v>
       </c>
       <c r="J106">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K106" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:11">
@@ -13450,22 +13483,25 @@
         <v>188</v>
       </c>
       <c r="E107">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="F107">
-        <v>188</v>
+        <v>32</v>
       </c>
       <c r="G107" s="1">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="H107" s="1">
-        <v>100</v>
+        <v>17</v>
+      </c>
+      <c r="I107" s="2">
+        <v>7.3</v>
       </c>
       <c r="J107">
-        <v>188</v>
+        <v>0</v>
       </c>
       <c r="K107" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:11">
@@ -13482,22 +13518,25 @@
         <v>39</v>
       </c>
       <c r="E108">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F108">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="G108" s="1">
-        <v>0</v>
+        <v>56.4</v>
       </c>
       <c r="H108" s="1">
-        <v>100</v>
+        <v>43.6</v>
+      </c>
+      <c r="I108" s="2">
+        <v>6.5</v>
       </c>
       <c r="J108">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K108" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:11">
@@ -13514,22 +13553,25 @@
         <v>36</v>
       </c>
       <c r="E109">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F109">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="G109" s="1">
-        <v>0</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="H109" s="1">
-        <v>100</v>
+        <v>13.9</v>
+      </c>
+      <c r="I109" s="2">
+        <v>6.9</v>
       </c>
       <c r="J109">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K109" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:11">
@@ -13546,22 +13588,25 @@
         <v>30</v>
       </c>
       <c r="E110">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F110">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="G110" s="1">
-        <v>0</v>
+        <v>93.3</v>
       </c>
       <c r="H110" s="1">
-        <v>100</v>
+        <v>6.7</v>
+      </c>
+      <c r="I110" s="2">
+        <v>6.8</v>
       </c>
       <c r="J110">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K110" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111" spans="1:11">
@@ -13575,22 +13620,25 @@
         <v>105</v>
       </c>
       <c r="E111">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="F111">
-        <v>105</v>
+        <v>24</v>
       </c>
       <c r="G111" s="1">
-        <v>0</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="H111" s="1">
-        <v>100</v>
+        <v>22.9</v>
+      </c>
+      <c r="I111" s="2">
+        <v>6.7</v>
       </c>
       <c r="J111">
-        <v>105</v>
+        <v>0</v>
       </c>
       <c r="K111" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112" spans="1:11">
@@ -13849,22 +13897,25 @@
         <v>27</v>
       </c>
       <c r="E119">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F119">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="G119" s="1">
-        <v>0</v>
+        <v>96.3</v>
       </c>
       <c r="H119" s="1">
-        <v>100</v>
+        <v>3.7</v>
+      </c>
+      <c r="I119" s="2">
+        <v>7.8</v>
       </c>
       <c r="J119">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="K119" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120" spans="1:11">
@@ -13881,22 +13932,25 @@
         <v>24</v>
       </c>
       <c r="E120">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F120">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="G120" s="1">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H120" s="1">
-        <v>100</v>
+        <v>25</v>
+      </c>
+      <c r="I120" s="2">
+        <v>7.7</v>
       </c>
       <c r="J120">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K120" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121" spans="1:11">
@@ -13913,22 +13967,25 @@
         <v>30</v>
       </c>
       <c r="E121">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="F121">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G121" s="1">
-        <v>0</v>
+        <v>96.7</v>
       </c>
       <c r="H121" s="1">
-        <v>100</v>
+        <v>3.3</v>
+      </c>
+      <c r="I121" s="2">
+        <v>7.6</v>
       </c>
       <c r="J121">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K121" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122" spans="1:11">
@@ -13945,22 +14002,25 @@
         <v>27</v>
       </c>
       <c r="E122">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F122">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="G122" s="1">
-        <v>0</v>
+        <v>77.8</v>
       </c>
       <c r="H122" s="1">
-        <v>100</v>
+        <v>22.2</v>
+      </c>
+      <c r="I122" s="2">
+        <v>7.6</v>
       </c>
       <c r="J122">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="K122" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123" spans="1:11">
@@ -13977,22 +14037,25 @@
         <v>36</v>
       </c>
       <c r="E123">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F123">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="G123" s="1">
-        <v>0</v>
+        <v>91.7</v>
       </c>
       <c r="H123" s="1">
-        <v>97.2</v>
+        <v>8.300000000000001</v>
+      </c>
+      <c r="I123" s="2">
+        <v>8.800000000000001</v>
       </c>
       <c r="J123">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K123" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124" spans="1:11">
@@ -14009,22 +14072,25 @@
         <v>33</v>
       </c>
       <c r="E124">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F124">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="G124" s="1">
-        <v>0</v>
+        <v>84.8</v>
       </c>
       <c r="H124" s="1">
-        <v>100</v>
+        <v>15.2</v>
+      </c>
+      <c r="I124" s="2">
+        <v>8.1</v>
       </c>
       <c r="J124">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K124" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125" spans="1:11">
@@ -14041,22 +14107,25 @@
         <v>12</v>
       </c>
       <c r="E125">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F125">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G125" s="1">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H125" s="1">
-        <v>100</v>
+        <v>25</v>
+      </c>
+      <c r="I125" s="2">
+        <v>8.1</v>
       </c>
       <c r="J125">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K125" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126" spans="1:11">
@@ -14070,22 +14139,25 @@
         <v>189</v>
       </c>
       <c r="E126">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="F126">
-        <v>188</v>
+        <v>25</v>
       </c>
       <c r="G126" s="1">
-        <v>0</v>
+        <v>86.8</v>
       </c>
       <c r="H126" s="1">
-        <v>99.5</v>
+        <v>13.2</v>
+      </c>
+      <c r="I126" s="2">
+        <v>8</v>
       </c>
       <c r="J126">
-        <v>189</v>
+        <v>0</v>
       </c>
       <c r="K126" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127" spans="1:11">
@@ -14647,22 +14719,25 @@
         <v>31</v>
       </c>
       <c r="E143">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="F143">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="G143" s="1">
-        <v>0</v>
+        <v>93.5</v>
       </c>
       <c r="H143" s="1">
-        <v>100</v>
+        <v>6.5</v>
+      </c>
+      <c r="I143" s="2">
+        <v>7.9</v>
       </c>
       <c r="J143">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K143" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:11">
@@ -14711,25 +14786,25 @@
         <v>126</v>
       </c>
       <c r="E145">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="F145">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="G145" s="1">
-        <v>63.5</v>
+        <v>86.5</v>
       </c>
       <c r="H145" s="1">
-        <v>36.5</v>
+        <v>13.5</v>
       </c>
       <c r="I145" s="2">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="J145">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K145" s="1">
-        <v>24.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146" spans="1:11">
@@ -14883,22 +14958,25 @@
         <v>28</v>
       </c>
       <c r="E150">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F150">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="G150" s="1">
-        <v>0</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H150" s="1">
-        <v>100</v>
+        <v>17.9</v>
+      </c>
+      <c r="I150" s="2">
+        <v>6.4</v>
       </c>
       <c r="J150">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K150" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151" spans="1:11">
@@ -14912,22 +14990,25 @@
         <v>28</v>
       </c>
       <c r="E151">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F151">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="G151" s="1">
-        <v>0</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H151" s="1">
-        <v>100</v>
+        <v>17.9</v>
+      </c>
+      <c r="I151" s="2">
+        <v>6.4</v>
       </c>
       <c r="J151">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K151" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:11">
@@ -14944,22 +15025,25 @@
         <v>27</v>
       </c>
       <c r="E152">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F152">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="G152" s="1">
-        <v>0</v>
+        <v>85.2</v>
       </c>
       <c r="H152" s="1">
-        <v>100</v>
+        <v>14.8</v>
+      </c>
+      <c r="I152" s="2">
+        <v>7.4</v>
       </c>
       <c r="J152">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="K152" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" spans="1:11">
@@ -14976,22 +15060,25 @@
         <v>24</v>
       </c>
       <c r="E153">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F153">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="G153" s="1">
-        <v>0</v>
+        <v>87.5</v>
       </c>
       <c r="H153" s="1">
-        <v>100</v>
+        <v>12.5</v>
+      </c>
+      <c r="I153" s="2">
+        <v>6.5</v>
       </c>
       <c r="J153">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K153" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154" spans="1:11">
@@ -15008,22 +15095,25 @@
         <v>34</v>
       </c>
       <c r="E154">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F154">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="G154" s="1">
-        <v>0</v>
+        <v>91.2</v>
       </c>
       <c r="H154" s="1">
-        <v>100</v>
+        <v>8.800000000000001</v>
+      </c>
+      <c r="I154" s="2">
+        <v>7.7</v>
       </c>
       <c r="J154">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K154" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="155" spans="1:11">
@@ -15040,22 +15130,25 @@
         <v>40</v>
       </c>
       <c r="E155">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F155">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="G155" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H155" s="1">
-        <v>97.5</v>
+        <v>7.5</v>
+      </c>
+      <c r="I155" s="2">
+        <v>7.8</v>
       </c>
       <c r="J155">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="K155" s="1">
-        <v>100</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="156" spans="1:11">
@@ -15072,22 +15165,25 @@
         <v>39</v>
       </c>
       <c r="E156">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F156">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="G156" s="1">
-        <v>0</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H156" s="1">
-        <v>100</v>
+        <v>5.1</v>
+      </c>
+      <c r="I156" s="2">
+        <v>9</v>
       </c>
       <c r="J156">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K156" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="157" spans="1:11">
@@ -15104,22 +15200,25 @@
         <v>30</v>
       </c>
       <c r="E157">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F157">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G157" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H157" s="1">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="I157" s="2">
+        <v>8</v>
       </c>
       <c r="J157">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K157" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158" spans="1:11">
@@ -15133,22 +15232,25 @@
         <v>194</v>
       </c>
       <c r="E158">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="F158">
-        <v>193</v>
+        <v>15</v>
       </c>
       <c r="G158" s="1">
-        <v>0</v>
+        <v>91.8</v>
       </c>
       <c r="H158" s="1">
-        <v>99.5</v>
+        <v>7.7</v>
+      </c>
+      <c r="I158" s="2">
+        <v>7.7</v>
       </c>
       <c r="J158">
-        <v>194</v>
+        <v>1</v>
       </c>
       <c r="K158" s="1">
-        <v>100</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="159" spans="1:11">
@@ -15719,22 +15821,25 @@
         <v>39</v>
       </c>
       <c r="E175">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="F175">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="G175" s="1">
-        <v>0</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="H175" s="1">
-        <v>100</v>
+        <v>25.6</v>
+      </c>
+      <c r="I175" s="2">
+        <v>6.4</v>
       </c>
       <c r="J175">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K175" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176" spans="1:11">
@@ -15888,25 +15993,25 @@
         <v>239</v>
       </c>
       <c r="E180">
-        <v>176</v>
+        <v>205</v>
       </c>
       <c r="F180">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="G180" s="1">
-        <v>73.59999999999999</v>
+        <v>85.8</v>
       </c>
       <c r="H180" s="1">
-        <v>26.4</v>
+        <v>14.2</v>
       </c>
       <c r="I180" s="2">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="J180">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K180" s="1">
-        <v>16.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="181" spans="1:11">
@@ -15923,22 +16028,25 @@
         <v>28</v>
       </c>
       <c r="E181">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F181">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="G181" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H181" s="1">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="I181" s="2">
+        <v>6.9</v>
       </c>
       <c r="J181">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K181" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182" spans="1:11">
@@ -15955,22 +16063,25 @@
         <v>33</v>
       </c>
       <c r="E182">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F182">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="G182" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H182" s="1">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="I182" s="2">
+        <v>7.5</v>
       </c>
       <c r="J182">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K182" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="183" spans="1:11">
@@ -15987,22 +16098,25 @@
         <v>33</v>
       </c>
       <c r="E183">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F183">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="G183" s="1">
-        <v>0</v>
+        <v>75.8</v>
       </c>
       <c r="H183" s="1">
-        <v>100</v>
+        <v>24.2</v>
+      </c>
+      <c r="I183" s="2">
+        <v>6.1</v>
       </c>
       <c r="J183">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="K183" s="1">
-        <v>100</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="184" spans="1:11">
@@ -16054,22 +16168,25 @@
         <v>12</v>
       </c>
       <c r="E185">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F185">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G185" s="1">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="H185" s="1">
-        <v>100</v>
+        <v>33.3</v>
+      </c>
+      <c r="I185" s="2">
+        <v>6</v>
       </c>
       <c r="J185">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K185" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="186" spans="1:11">
@@ -16083,25 +16200,25 @@
         <v>132</v>
       </c>
       <c r="E186">
-        <v>16</v>
+        <v>110</v>
       </c>
       <c r="F186">
-        <v>116</v>
+        <v>22</v>
       </c>
       <c r="G186" s="1">
-        <v>12.1</v>
+        <v>83.3</v>
       </c>
       <c r="H186" s="1">
-        <v>87.90000000000001</v>
+        <v>16.7</v>
       </c>
       <c r="I186" s="2">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
       <c r="J186">
-        <v>106</v>
+        <v>3</v>
       </c>
       <c r="K186" s="1">
-        <v>80.3</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="187" spans="1:11">
@@ -16182,22 +16299,25 @@
         <v>42</v>
       </c>
       <c r="E189">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="F189">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="G189" s="1">
-        <v>0</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="H189" s="1">
-        <v>100</v>
+        <v>2.4</v>
+      </c>
+      <c r="I189" s="2">
+        <v>8.699999999999999</v>
       </c>
       <c r="J189">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="K189" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190" spans="1:11">
@@ -16243,22 +16363,25 @@
         <v>146</v>
       </c>
       <c r="E191">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="F191">
-        <v>146</v>
+        <v>105</v>
       </c>
       <c r="G191" s="1">
-        <v>0</v>
+        <v>28.1</v>
       </c>
       <c r="H191" s="1">
-        <v>100</v>
+        <v>71.90000000000001</v>
+      </c>
+      <c r="I191" s="2">
+        <v>8.699999999999999</v>
       </c>
       <c r="J191">
-        <v>146</v>
+        <v>104</v>
       </c>
       <c r="K191" s="1">
-        <v>100</v>
+        <v>71.2</v>
       </c>
     </row>
     <row r="192" spans="1:11">
@@ -16549,22 +16672,25 @@
         <v>36</v>
       </c>
       <c r="E200">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F200">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="G200" s="1">
-        <v>0</v>
+        <v>47.2</v>
       </c>
       <c r="H200" s="1">
-        <v>100</v>
+        <v>52.8</v>
+      </c>
+      <c r="I200" s="2">
+        <v>5.3</v>
       </c>
       <c r="J200">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K200" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="201" spans="1:11">
@@ -16581,22 +16707,25 @@
         <v>39</v>
       </c>
       <c r="E201">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F201">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="G201" s="1">
-        <v>0</v>
+        <v>51.3</v>
       </c>
       <c r="H201" s="1">
-        <v>100</v>
+        <v>48.7</v>
+      </c>
+      <c r="I201" s="2">
+        <v>5.6</v>
       </c>
       <c r="J201">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K201" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="202" spans="1:11">
@@ -16613,22 +16742,25 @@
         <v>39</v>
       </c>
       <c r="E202">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F202">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="G202" s="1">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="H202" s="1">
-        <v>100</v>
+        <v>66.7</v>
+      </c>
+      <c r="I202" s="2">
+        <v>5.4</v>
       </c>
       <c r="J202">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K202" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="203" spans="1:11">
@@ -16645,22 +16777,25 @@
         <v>19</v>
       </c>
       <c r="E203">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F203">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G203" s="1">
-        <v>0</v>
+        <v>47.4</v>
       </c>
       <c r="H203" s="1">
-        <v>94.7</v>
+        <v>52.6</v>
+      </c>
+      <c r="I203" s="2">
+        <v>5.4</v>
       </c>
       <c r="J203">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K203" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="204" spans="1:11">
@@ -16674,22 +16809,25 @@
         <v>133</v>
       </c>
       <c r="E204">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="F204">
-        <v>132</v>
+        <v>74</v>
       </c>
       <c r="G204" s="1">
-        <v>0</v>
+        <v>44.4</v>
       </c>
       <c r="H204" s="1">
-        <v>99.2</v>
+        <v>55.6</v>
+      </c>
+      <c r="I204" s="2">
+        <v>5.4</v>
       </c>
       <c r="J204">
-        <v>133</v>
+        <v>0</v>
       </c>
       <c r="K204" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205" spans="1:11">
@@ -17129,10 +17267,10 @@
         <v>5.7</v>
       </c>
       <c r="J217">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K217" s="1">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="218" spans="1:11">
@@ -17336,10 +17474,10 @@
         <v>6.4</v>
       </c>
       <c r="J223">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K223" s="1">
-        <v>0.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="224" spans="1:11">
@@ -17790,22 +17928,25 @@
         <v>27</v>
       </c>
       <c r="E237">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F237">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="G237" s="1">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="H237" s="1">
-        <v>100</v>
+        <v>33.3</v>
+      </c>
+      <c r="I237" s="2">
+        <v>7.1</v>
       </c>
       <c r="J237">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="K237" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="238" spans="1:11">
@@ -17822,22 +17963,25 @@
         <v>24</v>
       </c>
       <c r="E238">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F238">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="G238" s="1">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H238" s="1">
-        <v>100</v>
+        <v>25</v>
+      </c>
+      <c r="I238" s="2">
+        <v>7.4</v>
       </c>
       <c r="J238">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K238" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="239" spans="1:11">
@@ -17918,22 +18062,25 @@
         <v>25</v>
       </c>
       <c r="E241">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F241">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="G241" s="1">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="H241" s="1">
-        <v>100</v>
+        <v>16</v>
+      </c>
+      <c r="I241" s="2">
+        <v>7.9</v>
       </c>
       <c r="J241">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K241" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="242" spans="1:11">
@@ -17982,25 +18129,25 @@
         <v>181</v>
       </c>
       <c r="E243">
-        <v>30</v>
+        <v>87</v>
       </c>
       <c r="F243">
-        <v>151</v>
+        <v>94</v>
       </c>
       <c r="G243" s="1">
-        <v>16.6</v>
+        <v>48.1</v>
       </c>
       <c r="H243" s="1">
-        <v>83.40000000000001</v>
+        <v>51.9</v>
       </c>
       <c r="I243" s="2">
-        <v>7</v>
+        <v>7.4</v>
       </c>
       <c r="J243">
-        <v>145</v>
+        <v>69</v>
       </c>
       <c r="K243" s="1">
-        <v>80.09999999999999</v>
+        <v>38.1</v>
       </c>
     </row>
     <row r="244" spans="1:11">
@@ -18017,22 +18164,25 @@
         <v>39</v>
       </c>
       <c r="E244">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F244">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="G244" s="1">
-        <v>0</v>
+        <v>56.4</v>
       </c>
       <c r="H244" s="1">
-        <v>97.40000000000001</v>
+        <v>43.6</v>
+      </c>
+      <c r="I244" s="2">
+        <v>5.8</v>
       </c>
       <c r="J244">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K244" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="245" spans="1:11">
@@ -18049,22 +18199,25 @@
         <v>39</v>
       </c>
       <c r="E245">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F245">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="G245" s="1">
-        <v>0</v>
+        <v>35.9</v>
       </c>
       <c r="H245" s="1">
-        <v>100</v>
+        <v>64.09999999999999</v>
+      </c>
+      <c r="I245" s="2">
+        <v>5.4</v>
       </c>
       <c r="J245">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K245" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="246" spans="1:11">
@@ -18081,22 +18234,25 @@
         <v>37</v>
       </c>
       <c r="E246">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F246">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="G246" s="1">
-        <v>0</v>
+        <v>40.5</v>
       </c>
       <c r="H246" s="1">
-        <v>100</v>
+        <v>59.5</v>
+      </c>
+      <c r="I246" s="2">
+        <v>5.6</v>
       </c>
       <c r="J246">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K246" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="247" spans="1:11">
@@ -18113,22 +18269,25 @@
         <v>19</v>
       </c>
       <c r="E247">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F247">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G247" s="1">
-        <v>0</v>
+        <v>47.4</v>
       </c>
       <c r="H247" s="1">
-        <v>94.7</v>
+        <v>52.6</v>
+      </c>
+      <c r="I247" s="2">
+        <v>6.1</v>
       </c>
       <c r="J247">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K247" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248" spans="1:11">
@@ -18145,22 +18304,25 @@
         <v>24</v>
       </c>
       <c r="E248">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F248">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="G248" s="1">
-        <v>0</v>
+        <v>70.8</v>
       </c>
       <c r="H248" s="1">
-        <v>100</v>
+        <v>29.2</v>
+      </c>
+      <c r="I248" s="2">
+        <v>6</v>
       </c>
       <c r="J248">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K248" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="249" spans="1:11">
@@ -18177,22 +18339,25 @@
         <v>30</v>
       </c>
       <c r="E249">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F249">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="G249" s="1">
-        <v>0</v>
+        <v>93.3</v>
       </c>
       <c r="H249" s="1">
-        <v>100</v>
+        <v>6.7</v>
+      </c>
+      <c r="I249" s="2">
+        <v>6.9</v>
       </c>
       <c r="J249">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K249" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="250" spans="1:11">
@@ -18206,22 +18371,25 @@
         <v>188</v>
       </c>
       <c r="E250">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="F250">
-        <v>186</v>
+        <v>83</v>
       </c>
       <c r="G250" s="1">
-        <v>0</v>
+        <v>55.9</v>
       </c>
       <c r="H250" s="1">
-        <v>98.90000000000001</v>
+        <v>44.1</v>
+      </c>
+      <c r="I250" s="2">
+        <v>6</v>
       </c>
       <c r="J250">
-        <v>188</v>
+        <v>0</v>
       </c>
       <c r="K250" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="251" spans="1:11">
@@ -19223,19 +19391,19 @@
         <v>38</v>
       </c>
       <c r="E17">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F17">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G17" s="1">
-        <v>78.90000000000001</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="H17" s="1">
-        <v>21.1</v>
+        <v>18.4</v>
       </c>
       <c r="I17" s="2">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="J17">
         <v>38</v>
@@ -19258,19 +19426,19 @@
         <v>38</v>
       </c>
       <c r="E18">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G18" s="1">
-        <v>92.09999999999999</v>
+        <v>84.2</v>
       </c>
       <c r="H18" s="1">
-        <v>7.9</v>
+        <v>15.8</v>
       </c>
       <c r="I18" s="2">
-        <v>8.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="J18">
         <v>38</v>
@@ -19290,16 +19458,16 @@
         <v>160</v>
       </c>
       <c r="E19">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F19">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G19" s="1">
-        <v>90</v>
+        <v>88.8</v>
       </c>
       <c r="H19" s="1">
-        <v>10</v>
+        <v>11.2</v>
       </c>
       <c r="I19" s="2">
         <v>7.9</v>
@@ -19771,19 +19939,19 @@
         <v>39</v>
       </c>
       <c r="E33">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F33">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G33" s="1">
-        <v>59</v>
+        <v>56.4</v>
       </c>
       <c r="H33" s="1">
-        <v>41</v>
+        <v>43.6</v>
       </c>
       <c r="I33" s="2">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="J33">
         <v>39</v>
@@ -19806,19 +19974,19 @@
         <v>39</v>
       </c>
       <c r="E34">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F34">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G34" s="1">
-        <v>64.09999999999999</v>
+        <v>61.5</v>
       </c>
       <c r="H34" s="1">
-        <v>35.9</v>
+        <v>38.5</v>
       </c>
       <c r="I34" s="2">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="J34">
         <v>39</v>
@@ -19841,16 +20009,16 @@
         <v>37</v>
       </c>
       <c r="E35">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F35">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G35" s="1">
-        <v>54.1</v>
+        <v>40.5</v>
       </c>
       <c r="H35" s="1">
-        <v>45.9</v>
+        <v>59.5</v>
       </c>
       <c r="I35" s="2">
         <v>5.9</v>
@@ -19908,16 +20076,16 @@
         <v>170</v>
       </c>
       <c r="E37">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="F37">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G37" s="1">
-        <v>54.7</v>
+        <v>50.6</v>
       </c>
       <c r="H37" s="1">
-        <v>45.3</v>
+        <v>49.4</v>
       </c>
       <c r="I37" s="2">
         <v>6.4</v>
@@ -22118,16 +22286,16 @@
         <v>30</v>
       </c>
       <c r="E101">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F101">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G101" s="1">
-        <v>70</v>
+        <v>66.7</v>
       </c>
       <c r="H101" s="1">
-        <v>30</v>
+        <v>33.3</v>
       </c>
       <c r="I101" s="2">
         <v>6.5</v>
@@ -22165,7 +22333,7 @@
         <v>5.3</v>
       </c>
       <c r="I102" s="2">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J102">
         <v>38</v>
@@ -22188,19 +22356,19 @@
         <v>25</v>
       </c>
       <c r="E103">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F103">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G103" s="1">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="H103" s="1">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I103" s="2">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="J103">
         <v>25</v>
@@ -22223,19 +22391,19 @@
         <v>31</v>
       </c>
       <c r="E104">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F104">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G104" s="1">
-        <v>83.90000000000001</v>
+        <v>90.3</v>
       </c>
       <c r="H104" s="1">
-        <v>16.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I104" s="2">
-        <v>7</v>
+        <v>7.7</v>
       </c>
       <c r="J104">
         <v>31</v>
@@ -22258,19 +22426,19 @@
         <v>36</v>
       </c>
       <c r="E105">
+        <v>27</v>
+      </c>
+      <c r="F105">
+        <v>9</v>
+      </c>
+      <c r="G105" s="1">
+        <v>75</v>
+      </c>
+      <c r="H105" s="1">
         <v>25</v>
       </c>
-      <c r="F105">
-        <v>11</v>
-      </c>
-      <c r="G105" s="1">
-        <v>69.40000000000001</v>
-      </c>
-      <c r="H105" s="1">
-        <v>30.6</v>
-      </c>
       <c r="I105" s="2">
-        <v>6.2</v>
+        <v>6.9</v>
       </c>
       <c r="J105">
         <v>36</v>
@@ -22305,7 +22473,7 @@
         <v>10.7</v>
       </c>
       <c r="I106" s="2">
-        <v>7.9</v>
+        <v>7.4</v>
       </c>
       <c r="J106">
         <v>28</v>
@@ -22325,19 +22493,19 @@
         <v>188</v>
       </c>
       <c r="E107">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F107">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G107" s="1">
-        <v>81.90000000000001</v>
+        <v>83</v>
       </c>
       <c r="H107" s="1">
-        <v>18.1</v>
+        <v>17</v>
       </c>
       <c r="I107" s="2">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="J107">
         <v>188</v>
@@ -22360,16 +22528,16 @@
         <v>39</v>
       </c>
       <c r="E108">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F108">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G108" s="1">
-        <v>53.8</v>
+        <v>56.4</v>
       </c>
       <c r="H108" s="1">
-        <v>46.2</v>
+        <v>43.6</v>
       </c>
       <c r="I108" s="2">
         <v>6.4</v>
@@ -22395,19 +22563,19 @@
         <v>36</v>
       </c>
       <c r="E109">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F109">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G109" s="1">
-        <v>88.90000000000001</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="H109" s="1">
-        <v>11.1</v>
+        <v>13.9</v>
       </c>
       <c r="I109" s="2">
-        <v>8.4</v>
+        <v>7.8</v>
       </c>
       <c r="J109">
         <v>36</v>
@@ -22442,7 +22610,7 @@
         <v>6.7</v>
       </c>
       <c r="I110" s="2">
-        <v>8.699999999999999</v>
+        <v>8</v>
       </c>
       <c r="J110">
         <v>30</v>
@@ -22474,7 +22642,7 @@
         <v>22.9</v>
       </c>
       <c r="I111" s="2">
-        <v>7.8</v>
+        <v>7.4</v>
       </c>
       <c r="J111">
         <v>105</v>
@@ -22739,19 +22907,19 @@
         <v>27</v>
       </c>
       <c r="E119">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F119">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G119" s="1">
-        <v>92.59999999999999</v>
+        <v>96.3</v>
       </c>
       <c r="H119" s="1">
-        <v>7.4</v>
+        <v>3.7</v>
       </c>
       <c r="I119" s="2">
-        <v>8.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J119">
         <v>27</v>
@@ -22774,19 +22942,19 @@
         <v>24</v>
       </c>
       <c r="E120">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F120">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G120" s="1">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H120" s="1">
-        <v>16.7</v>
+        <v>25</v>
       </c>
       <c r="I120" s="2">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="J120">
         <v>24</v>
@@ -22821,7 +22989,7 @@
         <v>3.3</v>
       </c>
       <c r="I121" s="2">
-        <v>8.699999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J121">
         <v>30</v>
@@ -22844,19 +23012,19 @@
         <v>27</v>
       </c>
       <c r="E122">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F122">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G122" s="1">
-        <v>81.5</v>
+        <v>77.8</v>
       </c>
       <c r="H122" s="1">
-        <v>18.5</v>
+        <v>22.2</v>
       </c>
       <c r="I122" s="2">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="J122">
         <v>27</v>
@@ -22882,16 +23050,16 @@
         <v>33</v>
       </c>
       <c r="F123">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G123" s="1">
         <v>91.7</v>
       </c>
       <c r="H123" s="1">
-        <v>5.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I123" s="2">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J123">
         <v>36</v>
@@ -22914,19 +23082,19 @@
         <v>33</v>
       </c>
       <c r="E124">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F124">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G124" s="1">
-        <v>72.7</v>
+        <v>84.8</v>
       </c>
       <c r="H124" s="1">
-        <v>27.3</v>
+        <v>15.2</v>
       </c>
       <c r="I124" s="2">
-        <v>8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J124">
         <v>33</v>
@@ -22949,19 +23117,19 @@
         <v>12</v>
       </c>
       <c r="E125">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F125">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G125" s="1">
-        <v>66.7</v>
+        <v>75</v>
       </c>
       <c r="H125" s="1">
-        <v>33.3</v>
+        <v>25</v>
       </c>
       <c r="I125" s="2">
-        <v>7.3</v>
+        <v>7.9</v>
       </c>
       <c r="J125">
         <v>12</v>
@@ -22981,19 +23149,19 @@
         <v>189</v>
       </c>
       <c r="E126">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F126">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G126" s="1">
-        <v>85.2</v>
+        <v>86.8</v>
       </c>
       <c r="H126" s="1">
-        <v>14.3</v>
+        <v>13.2</v>
       </c>
       <c r="I126" s="2">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J126">
         <v>189</v>
@@ -23567,19 +23735,19 @@
         <v>31</v>
       </c>
       <c r="E143">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F143">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G143" s="1">
-        <v>90.3</v>
+        <v>93.5</v>
       </c>
       <c r="H143" s="1">
-        <v>9.699999999999999</v>
+        <v>6.5</v>
       </c>
       <c r="I143" s="2">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
       <c r="J143">
         <v>31</v>
@@ -23634,19 +23802,19 @@
         <v>126</v>
       </c>
       <c r="E145">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F145">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G145" s="1">
-        <v>85.7</v>
+        <v>86.5</v>
       </c>
       <c r="H145" s="1">
-        <v>14.3</v>
+        <v>13.5</v>
       </c>
       <c r="I145" s="2">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="J145">
         <v>126</v>
@@ -23818,7 +23986,7 @@
         <v>17.9</v>
       </c>
       <c r="I150" s="2">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="J150">
         <v>28</v>
@@ -23850,7 +24018,7 @@
         <v>17.9</v>
       </c>
       <c r="I151" s="2">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="J151">
         <v>28</v>
@@ -23873,19 +24041,19 @@
         <v>27</v>
       </c>
       <c r="E152">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F152">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G152" s="1">
-        <v>77.8</v>
+        <v>85.2</v>
       </c>
       <c r="H152" s="1">
-        <v>22.2</v>
+        <v>14.8</v>
       </c>
       <c r="I152" s="2">
-        <v>8.4</v>
+        <v>8</v>
       </c>
       <c r="J152">
         <v>27</v>
@@ -23908,19 +24076,19 @@
         <v>24</v>
       </c>
       <c r="E153">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F153">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G153" s="1">
-        <v>91.7</v>
+        <v>87.5</v>
       </c>
       <c r="H153" s="1">
-        <v>8.300000000000001</v>
+        <v>12.5</v>
       </c>
       <c r="I153" s="2">
-        <v>8.9</v>
+        <v>7.9</v>
       </c>
       <c r="J153">
         <v>24</v>
@@ -23955,7 +24123,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="I154" s="2">
-        <v>9.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="J154">
         <v>34</v>
@@ -23990,7 +24158,7 @@
         <v>7.5</v>
       </c>
       <c r="I155" s="2">
-        <v>9.5</v>
+        <v>8.9</v>
       </c>
       <c r="J155">
         <v>40</v>
@@ -24013,19 +24181,19 @@
         <v>39</v>
       </c>
       <c r="E156">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F156">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G156" s="1">
-        <v>92.3</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H156" s="1">
-        <v>7.7</v>
+        <v>5.1</v>
       </c>
       <c r="I156" s="2">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J156">
         <v>39</v>
@@ -24048,19 +24216,19 @@
         <v>30</v>
       </c>
       <c r="E157">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F157">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G157" s="1">
-        <v>96.7</v>
+        <v>100</v>
       </c>
       <c r="H157" s="1">
-        <v>3.3</v>
+        <v>0</v>
       </c>
       <c r="I157" s="2">
-        <v>9.5</v>
+        <v>8.9</v>
       </c>
       <c r="J157">
         <v>30</v>
@@ -24080,19 +24248,19 @@
         <v>194</v>
       </c>
       <c r="E158">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F158">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G158" s="1">
-        <v>90.2</v>
+        <v>91.8</v>
       </c>
       <c r="H158" s="1">
-        <v>9.300000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="I158" s="2">
-        <v>9.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="J158">
         <v>194</v>
@@ -24669,16 +24837,16 @@
         <v>39</v>
       </c>
       <c r="E175">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F175">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G175" s="1">
-        <v>82.09999999999999</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="H175" s="1">
-        <v>17.9</v>
+        <v>25.6</v>
       </c>
       <c r="I175" s="2">
         <v>6.7</v>
@@ -24841,16 +25009,16 @@
         <v>239</v>
       </c>
       <c r="E180">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F180">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G180" s="1">
-        <v>87</v>
+        <v>85.8</v>
       </c>
       <c r="H180" s="1">
-        <v>13</v>
+        <v>14.2</v>
       </c>
       <c r="I180" s="2">
         <v>7.6</v>
@@ -24888,7 +25056,7 @@
         <v>0</v>
       </c>
       <c r="I181" s="2">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="J181">
         <v>28</v>
@@ -24923,7 +25091,7 @@
         <v>0</v>
       </c>
       <c r="I182" s="2">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
       <c r="J182">
         <v>33</v>
@@ -24946,19 +25114,19 @@
         <v>33</v>
       </c>
       <c r="E183">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="F183">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G183" s="1">
-        <v>100</v>
+        <v>84.8</v>
       </c>
       <c r="H183" s="1">
-        <v>0</v>
+        <v>15.2</v>
       </c>
       <c r="I183" s="2">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="J183">
         <v>33</v>
@@ -25016,19 +25184,19 @@
         <v>12</v>
       </c>
       <c r="E185">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F185">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G185" s="1">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="H185" s="1">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="I185" s="2">
-        <v>7.6</v>
+        <v>6.9</v>
       </c>
       <c r="J185">
         <v>12</v>
@@ -25048,19 +25216,19 @@
         <v>132</v>
       </c>
       <c r="E186">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="F186">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="G186" s="1">
-        <v>92.40000000000001</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="H186" s="1">
-        <v>7.6</v>
+        <v>14.4</v>
       </c>
       <c r="I186" s="2">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="J186">
         <v>132</v>
@@ -25153,19 +25321,19 @@
         <v>42</v>
       </c>
       <c r="E189">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F189">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G189" s="1">
-        <v>92.90000000000001</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="H189" s="1">
-        <v>7.1</v>
+        <v>2.4</v>
       </c>
       <c r="I189" s="2">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="J189">
         <v>42</v>
@@ -25220,16 +25388,16 @@
         <v>146</v>
       </c>
       <c r="E191">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F191">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G191" s="1">
-        <v>86.3</v>
+        <v>87.7</v>
       </c>
       <c r="H191" s="1">
-        <v>13.7</v>
+        <v>12.3</v>
       </c>
       <c r="I191" s="2">
         <v>8.199999999999999</v>
@@ -25529,19 +25697,19 @@
         <v>36</v>
       </c>
       <c r="E200">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F200">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G200" s="1">
-        <v>61.1</v>
+        <v>47.2</v>
       </c>
       <c r="H200" s="1">
-        <v>38.9</v>
+        <v>52.8</v>
       </c>
       <c r="I200" s="2">
-        <v>6.1</v>
+        <v>5.7</v>
       </c>
       <c r="J200">
         <v>36</v>
@@ -25564,19 +25732,19 @@
         <v>39</v>
       </c>
       <c r="E201">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F201">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="G201" s="1">
-        <v>74.40000000000001</v>
+        <v>51.3</v>
       </c>
       <c r="H201" s="1">
-        <v>25.6</v>
+        <v>48.7</v>
       </c>
       <c r="I201" s="2">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="J201">
         <v>39</v>
@@ -25599,19 +25767,19 @@
         <v>39</v>
       </c>
       <c r="E202">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F202">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G202" s="1">
-        <v>48.7</v>
+        <v>33.3</v>
       </c>
       <c r="H202" s="1">
-        <v>51.3</v>
+        <v>66.7</v>
       </c>
       <c r="I202" s="2">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="J202">
         <v>39</v>
@@ -25634,19 +25802,19 @@
         <v>19</v>
       </c>
       <c r="E203">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F203">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G203" s="1">
-        <v>73.7</v>
+        <v>47.4</v>
       </c>
       <c r="H203" s="1">
-        <v>21.1</v>
+        <v>52.6</v>
       </c>
       <c r="I203" s="2">
-        <v>6.4</v>
+        <v>5.8</v>
       </c>
       <c r="J203">
         <v>19</v>
@@ -25666,19 +25834,19 @@
         <v>133</v>
       </c>
       <c r="E204">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="F204">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="G204" s="1">
-        <v>63.2</v>
+        <v>44.4</v>
       </c>
       <c r="H204" s="1">
-        <v>36.1</v>
+        <v>55.6</v>
       </c>
       <c r="I204" s="2">
-        <v>5.9</v>
+        <v>5.6</v>
       </c>
       <c r="J204">
         <v>133</v>
@@ -26794,19 +26962,19 @@
         <v>27</v>
       </c>
       <c r="E237">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F237">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G237" s="1">
-        <v>81.5</v>
+        <v>66.7</v>
       </c>
       <c r="H237" s="1">
-        <v>18.5</v>
+        <v>33.3</v>
       </c>
       <c r="I237" s="2">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="J237">
         <v>27</v>
@@ -26829,19 +26997,19 @@
         <v>24</v>
       </c>
       <c r="E238">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F238">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G238" s="1">
-        <v>83.3</v>
+        <v>75</v>
       </c>
       <c r="H238" s="1">
-        <v>16.7</v>
+        <v>25</v>
       </c>
       <c r="I238" s="2">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="J238">
         <v>24</v>
@@ -26934,19 +27102,19 @@
         <v>25</v>
       </c>
       <c r="E241">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F241">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G241" s="1">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="H241" s="1">
+        <v>16</v>
+      </c>
+      <c r="I241" s="2">
         <v>8</v>
-      </c>
-      <c r="I241" s="2">
-        <v>7.8</v>
       </c>
       <c r="J241">
         <v>25</v>
@@ -27001,16 +27169,16 @@
         <v>181</v>
       </c>
       <c r="E243">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="F243">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G243" s="1">
-        <v>86.7</v>
+        <v>82.3</v>
       </c>
       <c r="H243" s="1">
-        <v>13.3</v>
+        <v>17.7</v>
       </c>
       <c r="I243" s="2">
         <v>7.7</v>
@@ -27036,19 +27204,19 @@
         <v>39</v>
       </c>
       <c r="E244">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F244">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G244" s="1">
-        <v>59</v>
+        <v>56.4</v>
       </c>
       <c r="H244" s="1">
-        <v>41</v>
+        <v>43.6</v>
       </c>
       <c r="I244" s="2">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
       <c r="J244">
         <v>39</v>
@@ -27071,19 +27239,19 @@
         <v>39</v>
       </c>
       <c r="E245">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F245">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G245" s="1">
-        <v>53.8</v>
+        <v>35.9</v>
       </c>
       <c r="H245" s="1">
-        <v>46.2</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="I245" s="2">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="J245">
         <v>39</v>
@@ -27106,19 +27274,19 @@
         <v>37</v>
       </c>
       <c r="E246">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F246">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G246" s="1">
-        <v>35.1</v>
+        <v>40.5</v>
       </c>
       <c r="H246" s="1">
-        <v>64.90000000000001</v>
+        <v>59.5</v>
       </c>
       <c r="I246" s="2">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="J246">
         <v>37</v>
@@ -27141,19 +27309,19 @@
         <v>19</v>
       </c>
       <c r="E247">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F247">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G247" s="1">
-        <v>73.7</v>
+        <v>47.4</v>
       </c>
       <c r="H247" s="1">
-        <v>21.1</v>
+        <v>52.6</v>
       </c>
       <c r="I247" s="2">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="J247">
         <v>19</v>
@@ -27176,19 +27344,19 @@
         <v>24</v>
       </c>
       <c r="E248">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F248">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G248" s="1">
-        <v>79.2</v>
+        <v>70.8</v>
       </c>
       <c r="H248" s="1">
-        <v>20.8</v>
+        <v>29.2</v>
       </c>
       <c r="I248" s="2">
-        <v>6.9</v>
+        <v>6.5</v>
       </c>
       <c r="J248">
         <v>24</v>
@@ -27223,7 +27391,7 @@
         <v>6.7</v>
       </c>
       <c r="I249" s="2">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="J249">
         <v>30</v>
@@ -27243,19 +27411,19 @@
         <v>188</v>
       </c>
       <c r="E250">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="F250">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="G250" s="1">
-        <v>62.8</v>
+        <v>55.9</v>
       </c>
       <c r="H250" s="1">
-        <v>36.7</v>
+        <v>44.1</v>
       </c>
       <c r="I250" s="2">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="J250">
         <v>188</v>

</xml_diff>

<commit_message>
Estadisticos Tercer Parcial Socio
</commit_message>
<xml_diff>
--- a/DetalleXDocente20231.xlsx
+++ b/DetalleXDocente20231.xlsx
@@ -2688,15 +2688,27 @@
         <v>124</v>
       </c>
       <c r="D56">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F56">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="G56" s="1">
+        <v>95</v>
+      </c>
+      <c r="H56" s="1">
+        <v>5</v>
+      </c>
+      <c r="I56" s="2">
+        <v>9.800000000000001</v>
       </c>
       <c r="J56">
+        <v>0</v>
+      </c>
+      <c r="K56" s="1">
         <v>0</v>
       </c>
     </row>
@@ -2778,22 +2790,22 @@
         <v>101</v>
       </c>
       <c r="D59">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="E59">
-        <v>108</v>
+        <v>146</v>
       </c>
       <c r="F59">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G59" s="1">
-        <v>47.4</v>
+        <v>54.5</v>
       </c>
       <c r="H59" s="1">
-        <v>52.6</v>
+        <v>45.5</v>
       </c>
       <c r="I59" s="2">
-        <v>6.1</v>
+        <v>6.6</v>
       </c>
       <c r="J59">
         <v>0</v>
@@ -4265,15 +4277,27 @@
         <v>125</v>
       </c>
       <c r="D102">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E102">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="F102">
         <v>0</v>
       </c>
+      <c r="G102" s="1">
+        <v>100</v>
+      </c>
+      <c r="H102" s="1">
+        <v>0</v>
+      </c>
+      <c r="I102" s="2">
+        <v>10</v>
+      </c>
       <c r="J102">
+        <v>0</v>
+      </c>
+      <c r="K102" s="1">
         <v>0</v>
       </c>
     </row>
@@ -4495,22 +4519,22 @@
         <v>101</v>
       </c>
       <c r="D109">
-        <v>188</v>
+        <v>227</v>
       </c>
       <c r="E109">
-        <v>154</v>
+        <v>193</v>
       </c>
       <c r="F109">
         <v>34</v>
       </c>
       <c r="G109" s="1">
-        <v>81.90000000000001</v>
+        <v>85</v>
       </c>
       <c r="H109" s="1">
-        <v>18.1</v>
+        <v>15</v>
       </c>
       <c r="I109" s="2">
-        <v>7.1</v>
+        <v>7.5</v>
       </c>
       <c r="J109">
         <v>0</v>
@@ -4565,15 +4589,27 @@
         <v>115</v>
       </c>
       <c r="D111">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="E111">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F111">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="G111" s="1">
+        <v>75.7</v>
+      </c>
+      <c r="H111" s="1">
+        <v>24.3</v>
+      </c>
+      <c r="I111" s="2">
+        <v>8.800000000000001</v>
       </c>
       <c r="J111">
+        <v>0</v>
+      </c>
+      <c r="K111" s="1">
         <v>0</v>
       </c>
     </row>
@@ -4655,22 +4691,22 @@
         <v>101</v>
       </c>
       <c r="D114">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="E114">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="F114">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="G114" s="1">
-        <v>77.09999999999999</v>
+        <v>76.8</v>
       </c>
       <c r="H114" s="1">
-        <v>22.9</v>
+        <v>23.2</v>
       </c>
       <c r="I114" s="2">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="J114">
         <v>0</v>
@@ -5002,15 +5038,27 @@
         <v>116</v>
       </c>
       <c r="D124">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E124">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F124">
         <v>0</v>
       </c>
+      <c r="G124" s="1">
+        <v>100</v>
+      </c>
+      <c r="H124" s="1">
+        <v>0</v>
+      </c>
+      <c r="I124" s="2">
+        <v>10</v>
+      </c>
       <c r="J124">
+        <v>0</v>
+      </c>
+      <c r="K124" s="1">
         <v>0</v>
       </c>
     </row>
@@ -5197,22 +5245,22 @@
         <v>101</v>
       </c>
       <c r="D130">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="E130">
-        <v>163</v>
+        <v>182</v>
       </c>
       <c r="F130">
         <v>27</v>
       </c>
       <c r="G130" s="1">
-        <v>85.8</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="H130" s="1">
-        <v>14.2</v>
+        <v>12.9</v>
       </c>
       <c r="I130" s="2">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J130">
         <v>0</v>
@@ -5885,15 +5933,27 @@
         <v>123</v>
       </c>
       <c r="D150">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="E150">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="F150">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="G150" s="1">
+        <v>85.3</v>
+      </c>
+      <c r="H150" s="1">
+        <v>14.7</v>
+      </c>
+      <c r="I150" s="2">
+        <v>9.300000000000001</v>
       </c>
       <c r="J150">
+        <v>0</v>
+      </c>
+      <c r="K150" s="1">
         <v>0</v>
       </c>
     </row>
@@ -6010,22 +6070,22 @@
         <v>101</v>
       </c>
       <c r="D154">
-        <v>102</v>
+        <v>136</v>
       </c>
       <c r="E154">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="F154">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G154" s="1">
-        <v>96.09999999999999</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="H154" s="1">
-        <v>3.9</v>
+        <v>6.6</v>
       </c>
       <c r="I154" s="2">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="J154">
         <v>0</v>
@@ -6561,15 +6621,27 @@
         <v>121</v>
       </c>
       <c r="D170">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E170">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F170">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="G170" s="1">
+        <v>85.2</v>
+      </c>
+      <c r="H170" s="1">
+        <v>14.8</v>
+      </c>
+      <c r="I170" s="2">
+        <v>9.300000000000001</v>
       </c>
       <c r="J170">
+        <v>0</v>
+      </c>
+      <c r="K170" s="1">
         <v>0</v>
       </c>
     </row>
@@ -6826,22 +6898,22 @@
         <v>101</v>
       </c>
       <c r="D178">
-        <v>279</v>
+        <v>306</v>
       </c>
       <c r="E178">
-        <v>193</v>
+        <v>216</v>
       </c>
       <c r="F178">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G178" s="1">
-        <v>69.2</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="H178" s="1">
-        <v>29</v>
+        <v>27.8</v>
       </c>
       <c r="I178" s="2">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="J178">
         <v>0</v>
@@ -6966,15 +7038,27 @@
         <v>114</v>
       </c>
       <c r="D182">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E182">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F182">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="G182" s="1">
+        <v>94.90000000000001</v>
+      </c>
+      <c r="H182" s="1">
+        <v>5.1</v>
+      </c>
+      <c r="I182" s="2">
+        <v>9.699999999999999</v>
       </c>
       <c r="J182">
+        <v>0</v>
+      </c>
+      <c r="K182" s="1">
         <v>0</v>
       </c>
     </row>
@@ -7126,22 +7210,22 @@
         <v>101</v>
       </c>
       <c r="D187">
-        <v>239</v>
+        <v>278</v>
       </c>
       <c r="E187">
-        <v>210</v>
+        <v>247</v>
       </c>
       <c r="F187">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G187" s="1">
-        <v>87.90000000000001</v>
+        <v>88.8</v>
       </c>
       <c r="H187" s="1">
-        <v>12.1</v>
+        <v>11.2</v>
       </c>
       <c r="I187" s="2">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
       <c r="J187">
         <v>0</v>
@@ -7540,15 +7624,27 @@
         <v>112</v>
       </c>
       <c r="D199">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="E199">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F199">
         <v>0</v>
       </c>
+      <c r="G199" s="1">
+        <v>100</v>
+      </c>
+      <c r="H199" s="1">
+        <v>0</v>
+      </c>
+      <c r="I199" s="2">
+        <v>10</v>
+      </c>
       <c r="J199">
+        <v>0</v>
+      </c>
+      <c r="K199" s="1">
         <v>0</v>
       </c>
     </row>
@@ -7630,22 +7726,22 @@
         <v>101</v>
       </c>
       <c r="D202">
-        <v>74</v>
+        <v>110</v>
       </c>
       <c r="E202">
-        <v>66</v>
+        <v>102</v>
       </c>
       <c r="F202">
         <v>8</v>
       </c>
       <c r="G202" s="1">
-        <v>89.2</v>
+        <v>92.7</v>
       </c>
       <c r="H202" s="1">
-        <v>10.8</v>
+        <v>7.3</v>
       </c>
       <c r="I202" s="2">
-        <v>7.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J202">
         <v>0</v>
@@ -7907,15 +8003,27 @@
         <v>113</v>
       </c>
       <c r="D210">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E210">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="F210">
         <v>0</v>
       </c>
+      <c r="G210" s="1">
+        <v>100</v>
+      </c>
+      <c r="H210" s="1">
+        <v>0</v>
+      </c>
+      <c r="I210" s="2">
+        <v>10</v>
+      </c>
       <c r="J210">
+        <v>0</v>
+      </c>
+      <c r="K210" s="1">
         <v>0</v>
       </c>
     </row>
@@ -7997,22 +8105,22 @@
         <v>101</v>
       </c>
       <c r="D213">
-        <v>133</v>
+        <v>172</v>
       </c>
       <c r="E213">
-        <v>84</v>
+        <v>123</v>
       </c>
       <c r="F213">
         <v>49</v>
       </c>
       <c r="G213" s="1">
-        <v>63.2</v>
+        <v>71.5</v>
       </c>
       <c r="H213" s="1">
-        <v>36.8</v>
+        <v>28.5</v>
       </c>
       <c r="I213" s="2">
-        <v>5.9</v>
+        <v>6.7</v>
       </c>
       <c r="J213">
         <v>0</v>
@@ -8172,15 +8280,27 @@
         <v>126</v>
       </c>
       <c r="D218">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E218">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F218">
         <v>0</v>
       </c>
+      <c r="G218" s="1">
+        <v>100</v>
+      </c>
+      <c r="H218" s="1">
+        <v>0</v>
+      </c>
+      <c r="I218" s="2">
+        <v>10</v>
+      </c>
       <c r="J218">
+        <v>0</v>
+      </c>
+      <c r="K218" s="1">
         <v>0</v>
       </c>
     </row>
@@ -8227,22 +8347,22 @@
         <v>101</v>
       </c>
       <c r="D220">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="E220">
-        <v>156</v>
+        <v>186</v>
       </c>
       <c r="F220">
         <v>12</v>
       </c>
       <c r="G220" s="1">
-        <v>92.90000000000001</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="H220" s="1">
-        <v>7.1</v>
+        <v>6.1</v>
       </c>
       <c r="I220" s="2">
-        <v>8.1</v>
+        <v>8.4</v>
       </c>
       <c r="J220">
         <v>0</v>
@@ -8976,15 +9096,27 @@
         <v>122</v>
       </c>
       <c r="D242">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E242">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F242">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G242" s="1">
+        <v>95.8</v>
+      </c>
+      <c r="H242" s="1">
+        <v>4.2</v>
+      </c>
+      <c r="I242" s="2">
+        <v>9.800000000000001</v>
       </c>
       <c r="J242">
+        <v>0</v>
+      </c>
+      <c r="K242" s="1">
         <v>0</v>
       </c>
     </row>
@@ -9136,22 +9268,22 @@
         <v>101</v>
       </c>
       <c r="D247">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="E247">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="F247">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G247" s="1">
-        <v>95</v>
+        <v>95.2</v>
       </c>
       <c r="H247" s="1">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="I247" s="2">
-        <v>7.6</v>
+        <v>8</v>
       </c>
       <c r="J247">
         <v>0</v>
@@ -11981,15 +12113,27 @@
         <v>124</v>
       </c>
       <c r="D56">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F56">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="G56" s="1">
+        <v>95</v>
+      </c>
+      <c r="H56" s="1">
+        <v>5</v>
+      </c>
+      <c r="I56" s="2">
+        <v>9.800000000000001</v>
       </c>
       <c r="J56">
+        <v>0</v>
+      </c>
+      <c r="K56" s="1">
         <v>0</v>
       </c>
     </row>
@@ -12071,22 +12215,22 @@
         <v>101</v>
       </c>
       <c r="D59">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="E59">
-        <v>124</v>
+        <v>162</v>
       </c>
       <c r="F59">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G59" s="1">
-        <v>54.4</v>
+        <v>60.4</v>
       </c>
       <c r="H59" s="1">
-        <v>45.6</v>
+        <v>39.6</v>
       </c>
       <c r="I59" s="2">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="J59">
         <v>0</v>
@@ -13558,15 +13702,27 @@
         <v>125</v>
       </c>
       <c r="D102">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E102">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="F102">
         <v>0</v>
       </c>
+      <c r="G102" s="1">
+        <v>100</v>
+      </c>
+      <c r="H102" s="1">
+        <v>0</v>
+      </c>
+      <c r="I102" s="2">
+        <v>10</v>
+      </c>
       <c r="J102">
+        <v>0</v>
+      </c>
+      <c r="K102" s="1">
         <v>0</v>
       </c>
     </row>
@@ -13788,22 +13944,22 @@
         <v>101</v>
       </c>
       <c r="D109">
-        <v>188</v>
+        <v>227</v>
       </c>
       <c r="E109">
-        <v>156</v>
+        <v>195</v>
       </c>
       <c r="F109">
         <v>32</v>
       </c>
       <c r="G109" s="1">
-        <v>83</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="H109" s="1">
-        <v>17</v>
+        <v>14.1</v>
       </c>
       <c r="I109" s="2">
-        <v>7.3</v>
+        <v>7.7</v>
       </c>
       <c r="J109">
         <v>0</v>
@@ -13858,15 +14014,27 @@
         <v>115</v>
       </c>
       <c r="D111">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="E111">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F111">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="G111" s="1">
+        <v>86.5</v>
+      </c>
+      <c r="H111" s="1">
+        <v>13.5</v>
+      </c>
+      <c r="I111" s="2">
+        <v>8.800000000000001</v>
       </c>
       <c r="J111">
+        <v>0</v>
+      </c>
+      <c r="K111" s="1">
         <v>0</v>
       </c>
     </row>
@@ -13948,22 +14116,22 @@
         <v>101</v>
       </c>
       <c r="D114">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="E114">
-        <v>81</v>
+        <v>113</v>
       </c>
       <c r="F114">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="G114" s="1">
-        <v>77.09999999999999</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="H114" s="1">
-        <v>22.9</v>
+        <v>20.4</v>
       </c>
       <c r="I114" s="2">
-        <v>6.7</v>
+        <v>7.3</v>
       </c>
       <c r="J114">
         <v>0</v>
@@ -14295,15 +14463,27 @@
         <v>116</v>
       </c>
       <c r="D124">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E124">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F124">
         <v>0</v>
       </c>
+      <c r="G124" s="1">
+        <v>100</v>
+      </c>
+      <c r="H124" s="1">
+        <v>0</v>
+      </c>
+      <c r="I124" s="2">
+        <v>10</v>
+      </c>
       <c r="J124">
+        <v>0</v>
+      </c>
+      <c r="K124" s="1">
         <v>0</v>
       </c>
     </row>
@@ -14490,22 +14670,22 @@
         <v>101</v>
       </c>
       <c r="D130">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="E130">
-        <v>165</v>
+        <v>184</v>
       </c>
       <c r="F130">
         <v>25</v>
       </c>
       <c r="G130" s="1">
-        <v>86.8</v>
+        <v>88</v>
       </c>
       <c r="H130" s="1">
-        <v>13.2</v>
+        <v>12</v>
       </c>
       <c r="I130" s="2">
-        <v>7.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J130">
         <v>0</v>
@@ -15178,15 +15358,27 @@
         <v>123</v>
       </c>
       <c r="D150">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="E150">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F150">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="G150" s="1">
+        <v>94.09999999999999</v>
+      </c>
+      <c r="H150" s="1">
+        <v>5.9</v>
+      </c>
+      <c r="I150" s="2">
+        <v>9.699999999999999</v>
       </c>
       <c r="J150">
+        <v>0</v>
+      </c>
+      <c r="K150" s="1">
         <v>0</v>
       </c>
     </row>
@@ -15303,22 +15495,22 @@
         <v>101</v>
       </c>
       <c r="D154">
-        <v>102</v>
+        <v>136</v>
       </c>
       <c r="E154">
-        <v>97</v>
+        <v>129</v>
       </c>
       <c r="F154">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G154" s="1">
-        <v>95.09999999999999</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H154" s="1">
-        <v>4.9</v>
+        <v>5.1</v>
       </c>
       <c r="I154" s="2">
-        <v>8.6</v>
+        <v>8.9</v>
       </c>
       <c r="J154">
         <v>0</v>
@@ -15854,15 +16046,27 @@
         <v>121</v>
       </c>
       <c r="D170">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E170">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F170">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="G170" s="1">
+        <v>85.2</v>
+      </c>
+      <c r="H170" s="1">
+        <v>14.8</v>
+      </c>
+      <c r="I170" s="2">
+        <v>9.300000000000001</v>
       </c>
       <c r="J170">
+        <v>0</v>
+      </c>
+      <c r="K170" s="1">
         <v>0</v>
       </c>
     </row>
@@ -16119,22 +16323,22 @@
         <v>101</v>
       </c>
       <c r="D178">
-        <v>279</v>
+        <v>306</v>
       </c>
       <c r="E178">
-        <v>217</v>
+        <v>240</v>
       </c>
       <c r="F178">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G178" s="1">
-        <v>77.8</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="H178" s="1">
-        <v>21.5</v>
+        <v>20.9</v>
       </c>
       <c r="I178" s="2">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="J178">
         <v>0</v>
@@ -16259,15 +16463,27 @@
         <v>114</v>
       </c>
       <c r="D182">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E182">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F182">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="G182" s="1">
+        <v>94.90000000000001</v>
+      </c>
+      <c r="H182" s="1">
+        <v>5.1</v>
+      </c>
+      <c r="I182" s="2">
+        <v>9.699999999999999</v>
       </c>
       <c r="J182">
+        <v>0</v>
+      </c>
+      <c r="K182" s="1">
         <v>0</v>
       </c>
     </row>
@@ -16419,22 +16635,22 @@
         <v>101</v>
       </c>
       <c r="D187">
-        <v>239</v>
+        <v>278</v>
       </c>
       <c r="E187">
-        <v>205</v>
+        <v>242</v>
       </c>
       <c r="F187">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G187" s="1">
-        <v>85.8</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="H187" s="1">
-        <v>14.2</v>
+        <v>12.9</v>
       </c>
       <c r="I187" s="2">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
       <c r="J187">
         <v>0</v>
@@ -16833,15 +17049,27 @@
         <v>112</v>
       </c>
       <c r="D199">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="E199">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F199">
         <v>0</v>
       </c>
+      <c r="G199" s="1">
+        <v>100</v>
+      </c>
+      <c r="H199" s="1">
+        <v>0</v>
+      </c>
+      <c r="I199" s="2">
+        <v>10</v>
+      </c>
       <c r="J199">
+        <v>0</v>
+      </c>
+      <c r="K199" s="1">
         <v>0</v>
       </c>
     </row>
@@ -16923,22 +17151,22 @@
         <v>101</v>
       </c>
       <c r="D202">
-        <v>74</v>
+        <v>110</v>
       </c>
       <c r="E202">
-        <v>67</v>
+        <v>103</v>
       </c>
       <c r="F202">
         <v>7</v>
       </c>
       <c r="G202" s="1">
-        <v>90.5</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="H202" s="1">
-        <v>9.5</v>
+        <v>6.4</v>
       </c>
       <c r="I202" s="2">
-        <v>7.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J202">
         <v>0</v>
@@ -17200,15 +17428,27 @@
         <v>113</v>
       </c>
       <c r="D210">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E210">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="F210">
         <v>0</v>
       </c>
+      <c r="G210" s="1">
+        <v>100</v>
+      </c>
+      <c r="H210" s="1">
+        <v>0</v>
+      </c>
+      <c r="I210" s="2">
+        <v>9.4</v>
+      </c>
       <c r="J210">
+        <v>0</v>
+      </c>
+      <c r="K210" s="1">
         <v>0</v>
       </c>
     </row>
@@ -17290,22 +17530,22 @@
         <v>101</v>
       </c>
       <c r="D213">
-        <v>133</v>
+        <v>172</v>
       </c>
       <c r="E213">
-        <v>59</v>
+        <v>98</v>
       </c>
       <c r="F213">
         <v>74</v>
       </c>
       <c r="G213" s="1">
-        <v>44.4</v>
+        <v>57</v>
       </c>
       <c r="H213" s="1">
-        <v>55.6</v>
+        <v>43</v>
       </c>
       <c r="I213" s="2">
-        <v>5.4</v>
+        <v>6.2</v>
       </c>
       <c r="J213">
         <v>0</v>
@@ -17465,15 +17705,27 @@
         <v>126</v>
       </c>
       <c r="D218">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E218">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F218">
         <v>0</v>
       </c>
+      <c r="G218" s="1">
+        <v>100</v>
+      </c>
+      <c r="H218" s="1">
+        <v>0</v>
+      </c>
+      <c r="I218" s="2">
+        <v>10</v>
+      </c>
       <c r="J218">
+        <v>0</v>
+      </c>
+      <c r="K218" s="1">
         <v>0</v>
       </c>
     </row>
@@ -17520,22 +17772,22 @@
         <v>101</v>
       </c>
       <c r="D220">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="E220">
-        <v>158</v>
+        <v>188</v>
       </c>
       <c r="F220">
         <v>10</v>
       </c>
       <c r="G220" s="1">
-        <v>94</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H220" s="1">
-        <v>6</v>
+        <v>5.1</v>
       </c>
       <c r="I220" s="2">
-        <v>8.199999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="J220">
         <v>0</v>
@@ -18269,15 +18521,27 @@
         <v>122</v>
       </c>
       <c r="D242">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E242">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F242">
         <v>0</v>
       </c>
+      <c r="G242" s="1">
+        <v>100</v>
+      </c>
+      <c r="H242" s="1">
+        <v>0</v>
+      </c>
+      <c r="I242" s="2">
+        <v>10</v>
+      </c>
       <c r="J242">
+        <v>0</v>
+      </c>
+      <c r="K242" s="1">
         <v>0</v>
       </c>
     </row>
@@ -18429,22 +18693,22 @@
         <v>101</v>
       </c>
       <c r="D247">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="E247">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="F247">
         <v>22</v>
       </c>
       <c r="G247" s="1">
-        <v>81.8</v>
+        <v>84.8</v>
       </c>
       <c r="H247" s="1">
-        <v>18.2</v>
+        <v>15.2</v>
       </c>
       <c r="I247" s="2">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="J247">
         <v>0</v>
@@ -21274,15 +21538,27 @@
         <v>124</v>
       </c>
       <c r="D56">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="F56">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="G56" s="1">
+        <v>95</v>
+      </c>
+      <c r="H56" s="1">
+        <v>5</v>
+      </c>
+      <c r="I56" s="2">
+        <v>9.800000000000001</v>
       </c>
       <c r="J56">
+        <v>0</v>
+      </c>
+      <c r="K56" s="1">
         <v>0</v>
       </c>
     </row>
@@ -21364,22 +21640,22 @@
         <v>101</v>
       </c>
       <c r="D59">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="E59">
-        <v>157</v>
+        <v>195</v>
       </c>
       <c r="F59">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G59" s="1">
-        <v>68.90000000000001</v>
+        <v>72.8</v>
       </c>
       <c r="H59" s="1">
-        <v>31.1</v>
+        <v>27.2</v>
       </c>
       <c r="I59" s="2">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="J59">
         <v>0</v>
@@ -22851,15 +23127,27 @@
         <v>125</v>
       </c>
       <c r="D102">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E102">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="F102">
         <v>0</v>
       </c>
+      <c r="G102" s="1">
+        <v>100</v>
+      </c>
+      <c r="H102" s="1">
+        <v>0</v>
+      </c>
+      <c r="I102" s="2">
+        <v>10</v>
+      </c>
       <c r="J102">
+        <v>0</v>
+      </c>
+      <c r="K102" s="1">
         <v>0</v>
       </c>
     </row>
@@ -23081,22 +23369,22 @@
         <v>101</v>
       </c>
       <c r="D109">
-        <v>188</v>
+        <v>227</v>
       </c>
       <c r="E109">
-        <v>186</v>
+        <v>225</v>
       </c>
       <c r="F109">
         <v>2</v>
       </c>
       <c r="G109" s="1">
-        <v>98.90000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="H109" s="1">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="I109" s="2">
-        <v>7.6</v>
+        <v>8</v>
       </c>
       <c r="J109">
         <v>0</v>
@@ -23151,15 +23439,27 @@
         <v>115</v>
       </c>
       <c r="D111">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="E111">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F111">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="G111" s="1">
+        <v>73</v>
+      </c>
+      <c r="H111" s="1">
+        <v>27</v>
+      </c>
+      <c r="I111" s="2">
+        <v>8.6</v>
       </c>
       <c r="J111">
+        <v>0</v>
+      </c>
+      <c r="K111" s="1">
         <v>0</v>
       </c>
     </row>
@@ -23241,22 +23541,22 @@
         <v>101</v>
       </c>
       <c r="D114">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="E114">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="F114">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G114" s="1">
-        <v>90.5</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="H114" s="1">
-        <v>9.5</v>
+        <v>14.1</v>
       </c>
       <c r="I114" s="2">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="J114">
         <v>0</v>
@@ -23588,15 +23888,27 @@
         <v>116</v>
       </c>
       <c r="D124">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E124">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F124">
         <v>0</v>
       </c>
+      <c r="G124" s="1">
+        <v>100</v>
+      </c>
+      <c r="H124" s="1">
+        <v>0</v>
+      </c>
+      <c r="I124" s="2">
+        <v>10</v>
+      </c>
       <c r="J124">
+        <v>0</v>
+      </c>
+      <c r="K124" s="1">
         <v>0</v>
       </c>
     </row>
@@ -23783,22 +24095,22 @@
         <v>101</v>
       </c>
       <c r="D130">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="E130">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="F130">
         <v>12</v>
       </c>
       <c r="G130" s="1">
-        <v>93.7</v>
+        <v>94.3</v>
       </c>
       <c r="H130" s="1">
-        <v>6.3</v>
+        <v>5.7</v>
       </c>
       <c r="I130" s="2">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J130">
         <v>0</v>
@@ -24471,15 +24783,27 @@
         <v>123</v>
       </c>
       <c r="D150">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="E150">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F150">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="G150" s="1">
+        <v>94.09999999999999</v>
+      </c>
+      <c r="H150" s="1">
+        <v>5.9</v>
+      </c>
+      <c r="I150" s="2">
+        <v>9.699999999999999</v>
       </c>
       <c r="J150">
+        <v>0</v>
+      </c>
+      <c r="K150" s="1">
         <v>0</v>
       </c>
     </row>
@@ -24596,22 +24920,22 @@
         <v>101</v>
       </c>
       <c r="D154">
-        <v>102</v>
+        <v>136</v>
       </c>
       <c r="E154">
-        <v>100</v>
+        <v>132</v>
       </c>
       <c r="F154">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G154" s="1">
-        <v>98</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="H154" s="1">
-        <v>2</v>
+        <v>2.9</v>
       </c>
       <c r="I154" s="2">
-        <v>8.6</v>
+        <v>8.9</v>
       </c>
       <c r="J154">
         <v>0</v>
@@ -25147,15 +25471,27 @@
         <v>121</v>
       </c>
       <c r="D170">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="E170">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F170">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="G170" s="1">
+        <v>85.2</v>
+      </c>
+      <c r="H170" s="1">
+        <v>14.8</v>
+      </c>
+      <c r="I170" s="2">
+        <v>9.300000000000001</v>
       </c>
       <c r="J170">
+        <v>0</v>
+      </c>
+      <c r="K170" s="1">
         <v>0</v>
       </c>
     </row>
@@ -25412,22 +25748,22 @@
         <v>101</v>
       </c>
       <c r="D178">
-        <v>279</v>
+        <v>306</v>
       </c>
       <c r="E178">
-        <v>229</v>
+        <v>252</v>
       </c>
       <c r="F178">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G178" s="1">
-        <v>82.09999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="H178" s="1">
-        <v>17.9</v>
+        <v>17.6</v>
       </c>
       <c r="I178" s="2">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="J178">
         <v>0</v>
@@ -25552,15 +25888,27 @@
         <v>114</v>
       </c>
       <c r="D182">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E182">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F182">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="G182" s="1">
+        <v>94.90000000000001</v>
+      </c>
+      <c r="H182" s="1">
+        <v>5.1</v>
+      </c>
+      <c r="I182" s="2">
+        <v>9.699999999999999</v>
       </c>
       <c r="J182">
+        <v>0</v>
+      </c>
+      <c r="K182" s="1">
         <v>0</v>
       </c>
     </row>
@@ -25712,22 +26060,22 @@
         <v>101</v>
       </c>
       <c r="D187">
-        <v>239</v>
+        <v>278</v>
       </c>
       <c r="E187">
-        <v>211</v>
+        <v>248</v>
       </c>
       <c r="F187">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G187" s="1">
-        <v>88.3</v>
+        <v>89.2</v>
       </c>
       <c r="H187" s="1">
-        <v>11.7</v>
+        <v>10.8</v>
       </c>
       <c r="I187" s="2">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
       <c r="J187">
         <v>0</v>
@@ -26126,15 +26474,27 @@
         <v>112</v>
       </c>
       <c r="D199">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="E199">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F199">
         <v>0</v>
       </c>
+      <c r="G199" s="1">
+        <v>100</v>
+      </c>
+      <c r="H199" s="1">
+        <v>0</v>
+      </c>
+      <c r="I199" s="2">
+        <v>10</v>
+      </c>
       <c r="J199">
+        <v>0</v>
+      </c>
+      <c r="K199" s="1">
         <v>0</v>
       </c>
     </row>
@@ -26216,22 +26576,22 @@
         <v>101</v>
       </c>
       <c r="D202">
-        <v>74</v>
+        <v>110</v>
       </c>
       <c r="E202">
-        <v>70</v>
+        <v>106</v>
       </c>
       <c r="F202">
         <v>4</v>
       </c>
       <c r="G202" s="1">
-        <v>94.59999999999999</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="H202" s="1">
-        <v>5.4</v>
+        <v>3.6</v>
       </c>
       <c r="I202" s="2">
-        <v>7.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J202">
         <v>0</v>
@@ -26493,15 +26853,27 @@
         <v>113</v>
       </c>
       <c r="D210">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E210">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F210">
-        <v>0</v>
+        <v>37</v>
+      </c>
+      <c r="G210" s="1">
+        <v>5.1</v>
+      </c>
+      <c r="H210" s="1">
+        <v>94.90000000000001</v>
+      </c>
+      <c r="I210" s="2">
+        <v>5.3</v>
       </c>
       <c r="J210">
+        <v>0</v>
+      </c>
+      <c r="K210" s="1">
         <v>0</v>
       </c>
     </row>
@@ -26583,22 +26955,22 @@
         <v>101</v>
       </c>
       <c r="D213">
-        <v>133</v>
+        <v>172</v>
       </c>
       <c r="E213">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F213">
-        <v>65</v>
+        <v>102</v>
       </c>
       <c r="G213" s="1">
-        <v>51.1</v>
+        <v>40.7</v>
       </c>
       <c r="H213" s="1">
-        <v>48.9</v>
+        <v>59.3</v>
       </c>
       <c r="I213" s="2">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="J213">
         <v>0</v>
@@ -26758,15 +27130,27 @@
         <v>126</v>
       </c>
       <c r="D218">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E218">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="F218">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G218" s="1">
+        <v>96.7</v>
+      </c>
+      <c r="H218" s="1">
+        <v>3.3</v>
+      </c>
+      <c r="I218" s="2">
+        <v>9.800000000000001</v>
       </c>
       <c r="J218">
+        <v>0</v>
+      </c>
+      <c r="K218" s="1">
         <v>0</v>
       </c>
     </row>
@@ -26813,22 +27197,22 @@
         <v>101</v>
       </c>
       <c r="D220">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="E220">
-        <v>161</v>
+        <v>190</v>
       </c>
       <c r="F220">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G220" s="1">
-        <v>95.8</v>
+        <v>96</v>
       </c>
       <c r="H220" s="1">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="I220" s="2">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="J220">
         <v>0</v>
@@ -27562,15 +27946,27 @@
         <v>122</v>
       </c>
       <c r="D242">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E242">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F242">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G242" s="1">
+        <v>95.8</v>
+      </c>
+      <c r="H242" s="1">
+        <v>4.2</v>
+      </c>
+      <c r="I242" s="2">
+        <v>9.800000000000001</v>
       </c>
       <c r="J242">
+        <v>0</v>
+      </c>
+      <c r="K242" s="1">
         <v>0</v>
       </c>
     </row>
@@ -27722,22 +28118,22 @@
         <v>101</v>
       </c>
       <c r="D247">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="E247">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="F247">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G247" s="1">
-        <v>84.3</v>
+        <v>86.2</v>
       </c>
       <c r="H247" s="1">
-        <v>15.7</v>
+        <v>13.8</v>
       </c>
       <c r="I247" s="2">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
       <c r="J247">
         <v>0</v>

</xml_diff>

<commit_message>
Estadisticos Tercer Parcial Socioemocionales
</commit_message>
<xml_diff>
--- a/DetalleXDocente20231.xlsx
+++ b/DetalleXDocente20231.xlsx
@@ -19693,7 +19693,7 @@
         <v>0</v>
       </c>
       <c r="I2" s="2">
-        <v>8.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -19728,7 +19728,7 @@
         <v>12</v>
       </c>
       <c r="I3" s="2">
-        <v>7.8</v>
+        <v>9.4</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -19763,7 +19763,7 @@
         <v>12.5</v>
       </c>
       <c r="I4" s="2">
-        <v>7.6</v>
+        <v>9.4</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -19798,7 +19798,7 @@
         <v>11.8</v>
       </c>
       <c r="I5" s="2">
-        <v>7.5</v>
+        <v>9.4</v>
       </c>
       <c r="J5">
         <v>0</v>
@@ -19833,7 +19833,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="2">
-        <v>7.7</v>
+        <v>10</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -19865,7 +19865,7 @@
         <v>6.9</v>
       </c>
       <c r="I7" s="2">
-        <v>7.9</v>
+        <v>9.6</v>
       </c>
       <c r="J7">
         <v>0</v>
@@ -19900,7 +19900,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="2">
-        <v>8.6</v>
+        <v>10</v>
       </c>
       <c r="J8">
         <v>0</v>
@@ -19935,7 +19935,7 @@
         <v>2.4</v>
       </c>
       <c r="I9" s="2">
-        <v>8.199999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -19970,7 +19970,7 @@
         <v>11.1</v>
       </c>
       <c r="I10" s="2">
-        <v>7.3</v>
+        <v>9.4</v>
       </c>
       <c r="J10">
         <v>0</v>
@@ -20005,7 +20005,7 @@
         <v>20.9</v>
       </c>
       <c r="I11" s="2">
-        <v>7.2</v>
+        <v>9</v>
       </c>
       <c r="J11">
         <v>0</v>
@@ -20040,7 +20040,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="2">
-        <v>8.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="J12">
         <v>0</v>
@@ -20075,7 +20075,7 @@
         <v>2.6</v>
       </c>
       <c r="I13" s="2">
-        <v>8.5</v>
+        <v>9.9</v>
       </c>
       <c r="J13">
         <v>0</v>
@@ -20107,7 +20107,7 @@
         <v>6.8</v>
       </c>
       <c r="I14" s="2">
-        <v>8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J14">
         <v>0</v>
@@ -20142,7 +20142,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="2">
-        <v>8.4</v>
+        <v>10</v>
       </c>
       <c r="J15">
         <v>0</v>
@@ -20177,7 +20177,7 @@
         <v>2.4</v>
       </c>
       <c r="I16" s="2">
-        <v>8.300000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="J16">
         <v>0</v>
@@ -20212,7 +20212,7 @@
         <v>5.3</v>
       </c>
       <c r="I17" s="2">
-        <v>7.7</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J17">
         <v>0</v>
@@ -20247,7 +20247,7 @@
         <v>7.9</v>
       </c>
       <c r="I18" s="2">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
       <c r="J18">
         <v>0</v>
@@ -20279,7 +20279,7 @@
         <v>3.8</v>
       </c>
       <c r="I19" s="2">
-        <v>8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J19">
         <v>0</v>
@@ -20314,7 +20314,7 @@
         <v>0</v>
       </c>
       <c r="I20" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J20">
         <v>0</v>
@@ -20349,7 +20349,7 @@
         <v>11.1</v>
       </c>
       <c r="I21" s="2">
-        <v>7.1</v>
+        <v>9.4</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -20384,7 +20384,7 @@
         <v>3.7</v>
       </c>
       <c r="I22" s="2">
-        <v>8.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J22">
         <v>0</v>
@@ -20419,7 +20419,7 @@
         <v>3.8</v>
       </c>
       <c r="I23" s="2">
-        <v>7.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J23">
         <v>0</v>
@@ -20451,7 +20451,7 @@
         <v>4.5</v>
       </c>
       <c r="I24" s="2">
-        <v>7.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J24">
         <v>0</v>
@@ -20486,7 +20486,7 @@
         <v>0</v>
       </c>
       <c r="I25" s="2">
-        <v>9.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="J25">
         <v>0</v>
@@ -20518,7 +20518,7 @@
         <v>0</v>
       </c>
       <c r="I26" s="2">
-        <v>9.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="J26">
         <v>0</v>
@@ -20553,7 +20553,7 @@
         <v>3.3</v>
       </c>
       <c r="I27" s="2">
-        <v>8.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J27">
         <v>0</v>
@@ -20588,7 +20588,7 @@
         <v>3.1</v>
       </c>
       <c r="I28" s="2">
-        <v>8.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J28">
         <v>0</v>
@@ -20623,7 +20623,7 @@
         <v>0</v>
       </c>
       <c r="I29" s="2">
-        <v>8.9</v>
+        <v>10</v>
       </c>
       <c r="J29">
         <v>0</v>
@@ -20658,7 +20658,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="2">
-        <v>9.6</v>
+        <v>10</v>
       </c>
       <c r="J30">
         <v>0</v>
@@ -20690,7 +20690,7 @@
         <v>1.5</v>
       </c>
       <c r="I31" s="2">
-        <v>8.9</v>
+        <v>9.9</v>
       </c>
       <c r="J31">
         <v>0</v>
@@ -20725,7 +20725,7 @@
         <v>27.8</v>
       </c>
       <c r="I32" s="2">
-        <v>6.6</v>
+        <v>8.6</v>
       </c>
       <c r="J32">
         <v>0</v>
@@ -20760,7 +20760,7 @@
         <v>15.4</v>
       </c>
       <c r="I33" s="2">
-        <v>6.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J33">
         <v>0</v>
@@ -20795,7 +20795,7 @@
         <v>23.1</v>
       </c>
       <c r="I34" s="2">
-        <v>6.7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J34">
         <v>0</v>
@@ -20830,7 +20830,7 @@
         <v>51.4</v>
       </c>
       <c r="I35" s="2">
-        <v>6</v>
+        <v>7.4</v>
       </c>
       <c r="J35">
         <v>0</v>
@@ -20865,7 +20865,7 @@
         <v>21.1</v>
       </c>
       <c r="I36" s="2">
-        <v>6.9</v>
+        <v>8.9</v>
       </c>
       <c r="J36">
         <v>0</v>
@@ -20897,7 +20897,7 @@
         <v>28.2</v>
       </c>
       <c r="I37" s="2">
-        <v>6.6</v>
+        <v>8.6</v>
       </c>
       <c r="J37">
         <v>0</v>
@@ -20932,7 +20932,7 @@
         <v>3.1</v>
       </c>
       <c r="I38" s="2">
-        <v>8.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J38">
         <v>0</v>
@@ -20967,7 +20967,7 @@
         <v>0</v>
       </c>
       <c r="I39" s="2">
-        <v>8.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="J39">
         <v>0</v>
@@ -21002,7 +21002,7 @@
         <v>3.6</v>
       </c>
       <c r="I40" s="2">
-        <v>7.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J40">
         <v>0</v>
@@ -21034,7 +21034,7 @@
         <v>2.2</v>
       </c>
       <c r="I41" s="2">
-        <v>8.199999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="J41">
         <v>0</v>
@@ -21069,7 +21069,7 @@
         <v>5.6</v>
       </c>
       <c r="I42" s="2">
-        <v>7.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J42">
         <v>0</v>
@@ -21104,7 +21104,7 @@
         <v>8</v>
       </c>
       <c r="I43" s="2">
-        <v>7.1</v>
+        <v>9.6</v>
       </c>
       <c r="J43">
         <v>0</v>
@@ -21136,7 +21136,7 @@
         <v>6.6</v>
       </c>
       <c r="I44" s="2">
-        <v>7.4</v>
+        <v>9.6</v>
       </c>
       <c r="J44">
         <v>0</v>
@@ -21171,7 +21171,7 @@
         <v>48.6</v>
       </c>
       <c r="I45" s="2">
-        <v>6.1</v>
+        <v>7.6</v>
       </c>
       <c r="J45">
         <v>0</v>
@@ -21206,7 +21206,7 @@
         <v>15.2</v>
       </c>
       <c r="I46" s="2">
-        <v>6.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J46">
         <v>0</v>
@@ -21241,7 +21241,7 @@
         <v>12.5</v>
       </c>
       <c r="I47" s="2">
-        <v>7.1</v>
+        <v>9.4</v>
       </c>
       <c r="J47">
         <v>0</v>
@@ -21276,7 +21276,7 @@
         <v>3.8</v>
       </c>
       <c r="I48" s="2">
-        <v>7.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J48">
         <v>0</v>
@@ -21311,7 +21311,7 @@
         <v>15.4</v>
       </c>
       <c r="I49" s="2">
-        <v>6.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J49">
         <v>0</v>
@@ -21343,7 +21343,7 @@
         <v>22.4</v>
       </c>
       <c r="I50" s="2">
-        <v>6.8</v>
+        <v>9</v>
       </c>
       <c r="J50">
         <v>0</v>
@@ -21378,7 +21378,7 @@
         <v>51.9</v>
       </c>
       <c r="I51" s="2">
-        <v>5.9</v>
+        <v>7.4</v>
       </c>
       <c r="J51">
         <v>0</v>
@@ -21413,7 +21413,7 @@
         <v>58.3</v>
       </c>
       <c r="I52" s="2">
-        <v>6</v>
+        <v>7.1</v>
       </c>
       <c r="J52">
         <v>0</v>
@@ -21448,7 +21448,7 @@
         <v>32.4</v>
       </c>
       <c r="I53" s="2">
-        <v>6.5</v>
+        <v>8.4</v>
       </c>
       <c r="J53">
         <v>0</v>
@@ -21483,7 +21483,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="I54" s="2">
-        <v>8.1</v>
+        <v>9.6</v>
       </c>
       <c r="J54">
         <v>0</v>
@@ -21518,7 +21518,7 @@
         <v>25</v>
       </c>
       <c r="I55" s="2">
-        <v>6.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J55">
         <v>0</v>
@@ -21588,7 +21588,7 @@
         <v>23.1</v>
       </c>
       <c r="I57" s="2">
-        <v>6.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J57">
         <v>0</v>
@@ -21623,7 +21623,7 @@
         <v>33.3</v>
       </c>
       <c r="I58" s="2">
-        <v>6.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J58">
         <v>0</v>
@@ -21655,7 +21655,7 @@
         <v>27.2</v>
       </c>
       <c r="I59" s="2">
-        <v>7</v>
+        <v>8.5</v>
       </c>
       <c r="J59">
         <v>0</v>
@@ -21690,7 +21690,7 @@
         <v>9.800000000000001</v>
       </c>
       <c r="I60" s="2">
-        <v>7.2</v>
+        <v>9.5</v>
       </c>
       <c r="J60">
         <v>0</v>
@@ -21725,7 +21725,7 @@
         <v>0</v>
       </c>
       <c r="I61" s="2">
-        <v>7.4</v>
+        <v>10</v>
       </c>
       <c r="J61">
         <v>0</v>
@@ -21757,7 +21757,7 @@
         <v>5.4</v>
       </c>
       <c r="I62" s="2">
-        <v>7.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J62">
         <v>0</v>
@@ -21792,7 +21792,7 @@
         <v>18.5</v>
       </c>
       <c r="I63" s="2">
-        <v>7.4</v>
+        <v>9.1</v>
       </c>
       <c r="J63">
         <v>0</v>
@@ -21827,7 +21827,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="I64" s="2">
-        <v>8.4</v>
+        <v>9.6</v>
       </c>
       <c r="J64">
         <v>0</v>
@@ -21862,7 +21862,7 @@
         <v>2.5</v>
       </c>
       <c r="I65" s="2">
-        <v>8.800000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="J65">
         <v>0</v>
@@ -21897,7 +21897,7 @@
         <v>5.1</v>
       </c>
       <c r="I66" s="2">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J66">
         <v>0</v>
@@ -21932,7 +21932,7 @@
         <v>15.4</v>
       </c>
       <c r="I67" s="2">
-        <v>7.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J67">
         <v>0</v>
@@ -21967,7 +21967,7 @@
         <v>3.1</v>
       </c>
       <c r="I68" s="2">
-        <v>8.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J68">
         <v>0</v>
@@ -22002,7 +22002,7 @@
         <v>0</v>
       </c>
       <c r="I69" s="2">
-        <v>8.199999999999999</v>
+        <v>10</v>
       </c>
       <c r="J69">
         <v>0</v>
@@ -22037,7 +22037,7 @@
         <v>10.7</v>
       </c>
       <c r="I70" s="2">
-        <v>8</v>
+        <v>9.5</v>
       </c>
       <c r="J70">
         <v>0</v>
@@ -22069,7 +22069,7 @@
         <v>7.8</v>
       </c>
       <c r="I71" s="2">
-        <v>8.199999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="J71">
         <v>0</v>
@@ -22104,7 +22104,7 @@
         <v>7.9</v>
       </c>
       <c r="I72" s="2">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
       <c r="J72">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>6.7</v>
       </c>
       <c r="I73" s="2">
-        <v>7.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J73">
         <v>0</v>
@@ -22174,7 +22174,7 @@
         <v>0</v>
       </c>
       <c r="I74" s="2">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="J74">
         <v>0</v>
@@ -22209,7 +22209,7 @@
         <v>12</v>
       </c>
       <c r="I75" s="2">
-        <v>8.4</v>
+        <v>9.4</v>
       </c>
       <c r="J75">
         <v>0</v>
@@ -22244,7 +22244,7 @@
         <v>0</v>
       </c>
       <c r="I76" s="2">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="J76">
         <v>0</v>
@@ -22279,7 +22279,7 @@
         <v>3.7</v>
       </c>
       <c r="I77" s="2">
-        <v>7.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J77">
         <v>0</v>
@@ -22314,7 +22314,7 @@
         <v>0</v>
       </c>
       <c r="I78" s="2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J78">
         <v>0</v>
@@ -22349,7 +22349,7 @@
         <v>18.8</v>
       </c>
       <c r="I79" s="2">
-        <v>7.1</v>
+        <v>9.1</v>
       </c>
       <c r="J79">
         <v>0</v>
@@ -22381,7 +22381,7 @@
         <v>5</v>
       </c>
       <c r="I80" s="2">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J80">
         <v>0</v>
@@ -22416,7 +22416,7 @@
         <v>50</v>
       </c>
       <c r="I81" s="2">
-        <v>5.7</v>
+        <v>7.5</v>
       </c>
       <c r="J81">
         <v>0</v>
@@ -22451,7 +22451,7 @@
         <v>38.5</v>
       </c>
       <c r="I82" s="2">
-        <v>5.8</v>
+        <v>8.1</v>
       </c>
       <c r="J82">
         <v>0</v>
@@ -22486,7 +22486,7 @@
         <v>38.5</v>
       </c>
       <c r="I83" s="2">
-        <v>6.1</v>
+        <v>8.1</v>
       </c>
       <c r="J83">
         <v>0</v>
@@ -22521,7 +22521,7 @@
         <v>45.9</v>
       </c>
       <c r="I84" s="2">
-        <v>5.8</v>
+        <v>7.7</v>
       </c>
       <c r="J84">
         <v>0</v>
@@ -22556,7 +22556,7 @@
         <v>26.3</v>
       </c>
       <c r="I85" s="2">
-        <v>6.3</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J85">
         <v>0</v>
@@ -22588,7 +22588,7 @@
         <v>41.2</v>
       </c>
       <c r="I86" s="2">
-        <v>5.9</v>
+        <v>8</v>
       </c>
       <c r="J86">
         <v>0</v>
@@ -22623,7 +22623,7 @@
         <v>0</v>
       </c>
       <c r="I87" s="2">
-        <v>7.4</v>
+        <v>10</v>
       </c>
       <c r="J87">
         <v>0</v>
@@ -22658,7 +22658,7 @@
         <v>7.1</v>
       </c>
       <c r="I88" s="2">
-        <v>7.4</v>
+        <v>9.6</v>
       </c>
       <c r="J88">
         <v>0</v>
@@ -22693,7 +22693,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="I89" s="2">
-        <v>7.1</v>
+        <v>9.6</v>
       </c>
       <c r="J89">
         <v>0</v>
@@ -22728,7 +22728,7 @@
         <v>18.2</v>
       </c>
       <c r="I90" s="2">
-        <v>6.7</v>
+        <v>9.1</v>
       </c>
       <c r="J90">
         <v>0</v>
@@ -22763,7 +22763,7 @@
         <v>0</v>
       </c>
       <c r="I91" s="2">
-        <v>7.7</v>
+        <v>10</v>
       </c>
       <c r="J91">
         <v>0</v>
@@ -22798,7 +22798,7 @@
         <v>5.3</v>
       </c>
       <c r="I92" s="2">
-        <v>7.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J92">
         <v>0</v>
@@ -22833,7 +22833,7 @@
         <v>0</v>
       </c>
       <c r="I93" s="2">
-        <v>6.9</v>
+        <v>10</v>
       </c>
       <c r="J93">
         <v>0</v>
@@ -22865,7 +22865,7 @@
         <v>6.5</v>
       </c>
       <c r="I94" s="2">
-        <v>7.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J94">
         <v>0</v>
@@ -22900,7 +22900,7 @@
         <v>0</v>
       </c>
       <c r="I95" s="2">
-        <v>6.6</v>
+        <v>10</v>
       </c>
       <c r="J95">
         <v>0</v>
@@ -22935,7 +22935,7 @@
         <v>13.9</v>
       </c>
       <c r="I96" s="2">
-        <v>7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J96">
         <v>0</v>
@@ -22970,7 +22970,7 @@
         <v>3.8</v>
       </c>
       <c r="I97" s="2">
-        <v>7.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J97">
         <v>0</v>
@@ -23005,7 +23005,7 @@
         <v>3.6</v>
       </c>
       <c r="I98" s="2">
-        <v>7.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J98">
         <v>0</v>
@@ -23040,7 +23040,7 @@
         <v>25</v>
       </c>
       <c r="I99" s="2">
-        <v>7.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J99">
         <v>0</v>
@@ -23075,7 +23075,7 @@
         <v>0</v>
       </c>
       <c r="I100" s="2">
-        <v>8.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="J100">
         <v>0</v>
@@ -23107,7 +23107,7 @@
         <v>7.1</v>
       </c>
       <c r="I101" s="2">
-        <v>7.4</v>
+        <v>9.6</v>
       </c>
       <c r="J101">
         <v>0</v>
@@ -23177,7 +23177,7 @@
         <v>3.3</v>
       </c>
       <c r="I103" s="2">
-        <v>6.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J103">
         <v>0</v>
@@ -23212,7 +23212,7 @@
         <v>0</v>
       </c>
       <c r="I104" s="2">
-        <v>8.4</v>
+        <v>10</v>
       </c>
       <c r="J104">
         <v>0</v>
@@ -23247,7 +23247,7 @@
         <v>4</v>
       </c>
       <c r="I105" s="2">
-        <v>7.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J105">
         <v>0</v>
@@ -23282,7 +23282,7 @@
         <v>0</v>
       </c>
       <c r="I106" s="2">
-        <v>7.8</v>
+        <v>10</v>
       </c>
       <c r="J106">
         <v>0</v>
@@ -23317,7 +23317,7 @@
         <v>0</v>
       </c>
       <c r="I107" s="2">
-        <v>7.6</v>
+        <v>10</v>
       </c>
       <c r="J107">
         <v>0</v>
@@ -23352,7 +23352,7 @@
         <v>0</v>
       </c>
       <c r="I108" s="2">
-        <v>7.4</v>
+        <v>10</v>
       </c>
       <c r="J108">
         <v>0</v>
@@ -23384,7 +23384,7 @@
         <v>0.9</v>
       </c>
       <c r="I109" s="2">
-        <v>8</v>
+        <v>9.9</v>
       </c>
       <c r="J109">
         <v>0</v>
@@ -23419,7 +23419,7 @@
         <v>17.9</v>
       </c>
       <c r="I110" s="2">
-        <v>6.7</v>
+        <v>9.1</v>
       </c>
       <c r="J110">
         <v>0</v>
@@ -23489,7 +23489,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="I112" s="2">
-        <v>8.1</v>
+        <v>9.6</v>
       </c>
       <c r="J112">
         <v>0</v>
@@ -23524,7 +23524,7 @@
         <v>0</v>
       </c>
       <c r="I113" s="2">
-        <v>8.4</v>
+        <v>10</v>
       </c>
       <c r="J113">
         <v>0</v>
@@ -23556,7 +23556,7 @@
         <v>14.1</v>
       </c>
       <c r="I114" s="2">
-        <v>8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J114">
         <v>0</v>
@@ -23591,7 +23591,7 @@
         <v>29.6</v>
       </c>
       <c r="I115" s="2">
-        <v>6.3</v>
+        <v>8.5</v>
       </c>
       <c r="J115">
         <v>0</v>
@@ -23626,7 +23626,7 @@
         <v>29.2</v>
       </c>
       <c r="I116" s="2">
-        <v>6.3</v>
+        <v>8.5</v>
       </c>
       <c r="J116">
         <v>0</v>
@@ -23661,7 +23661,7 @@
         <v>17.6</v>
       </c>
       <c r="I117" s="2">
-        <v>6.9</v>
+        <v>9.1</v>
       </c>
       <c r="J117">
         <v>0</v>
@@ -23696,7 +23696,7 @@
         <v>10</v>
       </c>
       <c r="I118" s="2">
-        <v>6.7</v>
+        <v>9.5</v>
       </c>
       <c r="J118">
         <v>0</v>
@@ -23731,7 +23731,7 @@
         <v>15.4</v>
       </c>
       <c r="I119" s="2">
-        <v>7.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J119">
         <v>0</v>
@@ -23766,7 +23766,7 @@
         <v>10</v>
       </c>
       <c r="I120" s="2">
-        <v>6.7</v>
+        <v>9.5</v>
       </c>
       <c r="J120">
         <v>0</v>
@@ -23798,7 +23798,7 @@
         <v>17.5</v>
       </c>
       <c r="I121" s="2">
-        <v>6.7</v>
+        <v>9</v>
       </c>
       <c r="J121">
         <v>0</v>
@@ -23833,7 +23833,7 @@
         <v>11.1</v>
       </c>
       <c r="I122" s="2">
-        <v>7.9</v>
+        <v>9.4</v>
       </c>
       <c r="J122">
         <v>0</v>
@@ -23868,7 +23868,7 @@
         <v>12.5</v>
       </c>
       <c r="I123" s="2">
-        <v>7.6</v>
+        <v>9.4</v>
       </c>
       <c r="J123">
         <v>0</v>
@@ -23938,7 +23938,7 @@
         <v>0</v>
       </c>
       <c r="I125" s="2">
-        <v>8.1</v>
+        <v>10</v>
       </c>
       <c r="J125">
         <v>0</v>
@@ -23973,7 +23973,7 @@
         <v>3.7</v>
       </c>
       <c r="I126" s="2">
-        <v>8.199999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J126">
         <v>0</v>
@@ -24008,7 +24008,7 @@
         <v>0</v>
       </c>
       <c r="I127" s="2">
-        <v>8.9</v>
+        <v>10</v>
       </c>
       <c r="J127">
         <v>0</v>
@@ -24043,7 +24043,7 @@
         <v>12.1</v>
       </c>
       <c r="I128" s="2">
-        <v>8.1</v>
+        <v>9.4</v>
       </c>
       <c r="J128">
         <v>0</v>
@@ -24078,7 +24078,7 @@
         <v>7.7</v>
       </c>
       <c r="I129" s="2">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
       <c r="J129">
         <v>0</v>
@@ -24110,7 +24110,7 @@
         <v>5.7</v>
       </c>
       <c r="I130" s="2">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J130">
         <v>0</v>
@@ -24145,7 +24145,7 @@
         <v>12.5</v>
       </c>
       <c r="I131" s="2">
-        <v>7</v>
+        <v>9.4</v>
       </c>
       <c r="J131">
         <v>0</v>
@@ -24177,7 +24177,7 @@
         <v>12.5</v>
       </c>
       <c r="I132" s="2">
-        <v>7</v>
+        <v>9.4</v>
       </c>
       <c r="J132">
         <v>0</v>
@@ -24212,7 +24212,7 @@
         <v>2.8</v>
       </c>
       <c r="I133" s="2">
-        <v>9</v>
+        <v>9.9</v>
       </c>
       <c r="J133">
         <v>0</v>
@@ -24247,7 +24247,7 @@
         <v>0</v>
       </c>
       <c r="I134" s="2">
-        <v>7.8</v>
+        <v>10</v>
       </c>
       <c r="J134">
         <v>0</v>
@@ -24282,7 +24282,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="I135" s="2">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
       <c r="J135">
         <v>0</v>
@@ -24317,7 +24317,7 @@
         <v>3.8</v>
       </c>
       <c r="I136" s="2">
-        <v>9.199999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J136">
         <v>0</v>
@@ -24352,7 +24352,7 @@
         <v>0</v>
       </c>
       <c r="I137" s="2">
-        <v>8.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="J137">
         <v>0</v>
@@ -24384,7 +24384,7 @@
         <v>3.3</v>
       </c>
       <c r="I138" s="2">
-        <v>8.5</v>
+        <v>9.9</v>
       </c>
       <c r="J138">
         <v>0</v>
@@ -24419,7 +24419,7 @@
         <v>12.8</v>
       </c>
       <c r="I139" s="2">
-        <v>6.7</v>
+        <v>9.4</v>
       </c>
       <c r="J139">
         <v>0</v>
@@ -24454,7 +24454,7 @@
         <v>20.8</v>
       </c>
       <c r="I140" s="2">
-        <v>6.9</v>
+        <v>9</v>
       </c>
       <c r="J140">
         <v>0</v>
@@ -24489,7 +24489,7 @@
         <v>25</v>
       </c>
       <c r="I141" s="2">
-        <v>6.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J141">
         <v>0</v>
@@ -24524,7 +24524,7 @@
         <v>16</v>
       </c>
       <c r="I142" s="2">
-        <v>8.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J142">
         <v>0</v>
@@ -24559,7 +24559,7 @@
         <v>7.7</v>
       </c>
       <c r="I143" s="2">
-        <v>8.199999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="J143">
         <v>0</v>
@@ -24591,7 +24591,7 @@
         <v>15.9</v>
       </c>
       <c r="I144" s="2">
-        <v>7.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J144">
         <v>0</v>
@@ -24626,7 +24626,7 @@
         <v>0</v>
       </c>
       <c r="I145" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J145">
         <v>0</v>
@@ -24661,7 +24661,7 @@
         <v>0</v>
       </c>
       <c r="I146" s="2">
-        <v>8.6</v>
+        <v>10</v>
       </c>
       <c r="J146">
         <v>0</v>
@@ -24696,7 +24696,7 @@
         <v>0</v>
       </c>
       <c r="I147" s="2">
-        <v>7.9</v>
+        <v>10</v>
       </c>
       <c r="J147">
         <v>0</v>
@@ -24731,7 +24731,7 @@
         <v>14.8</v>
       </c>
       <c r="I148" s="2">
-        <v>7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J148">
         <v>0</v>
@@ -24763,7 +24763,7 @@
         <v>3.2</v>
       </c>
       <c r="I149" s="2">
-        <v>7.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J149">
         <v>0</v>
@@ -24833,7 +24833,7 @@
         <v>2.3</v>
       </c>
       <c r="I151" s="2">
-        <v>8.300000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="J151">
         <v>0</v>
@@ -24868,7 +24868,7 @@
         <v>3.7</v>
       </c>
       <c r="I152" s="2">
-        <v>8.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J152">
         <v>0</v>
@@ -24903,7 +24903,7 @@
         <v>0</v>
       </c>
       <c r="I153" s="2">
-        <v>9.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="J153">
         <v>0</v>
@@ -24935,7 +24935,7 @@
         <v>2.9</v>
       </c>
       <c r="I154" s="2">
-        <v>8.9</v>
+        <v>9.9</v>
       </c>
       <c r="J154">
         <v>0</v>
@@ -24970,7 +24970,7 @@
         <v>17.9</v>
       </c>
       <c r="I155" s="2">
-        <v>7</v>
+        <v>9.1</v>
       </c>
       <c r="J155">
         <v>0</v>
@@ -25002,7 +25002,7 @@
         <v>17.9</v>
       </c>
       <c r="I156" s="2">
-        <v>7</v>
+        <v>9.1</v>
       </c>
       <c r="J156">
         <v>0</v>
@@ -25037,7 +25037,7 @@
         <v>22.2</v>
       </c>
       <c r="I157" s="2">
-        <v>7.4</v>
+        <v>8.9</v>
       </c>
       <c r="J157">
         <v>0</v>
@@ -25072,7 +25072,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="I158" s="2">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
       <c r="J158">
         <v>0</v>
@@ -25107,7 +25107,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="I159" s="2">
-        <v>8.4</v>
+        <v>9.6</v>
       </c>
       <c r="J159">
         <v>0</v>
@@ -25142,7 +25142,7 @@
         <v>5</v>
       </c>
       <c r="I160" s="2">
-        <v>8.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J160">
         <v>0</v>
@@ -25177,7 +25177,7 @@
         <v>5.1</v>
       </c>
       <c r="I161" s="2">
-        <v>9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J161">
         <v>0</v>
@@ -25212,7 +25212,7 @@
         <v>3.3</v>
       </c>
       <c r="I162" s="2">
-        <v>7.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J162">
         <v>0</v>
@@ -25244,7 +25244,7 @@
         <v>8.199999999999999</v>
       </c>
       <c r="I163" s="2">
-        <v>8.1</v>
+        <v>9.6</v>
       </c>
       <c r="J163">
         <v>0</v>
@@ -25279,7 +25279,7 @@
         <v>16.7</v>
       </c>
       <c r="I164" s="2">
-        <v>6.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J164">
         <v>0</v>
@@ -25314,7 +25314,7 @@
         <v>12.5</v>
       </c>
       <c r="I165" s="2">
-        <v>7.8</v>
+        <v>9.4</v>
       </c>
       <c r="J165">
         <v>0</v>
@@ -25349,7 +25349,7 @@
         <v>11.5</v>
       </c>
       <c r="I166" s="2">
-        <v>8.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="J166">
         <v>0</v>
@@ -25384,7 +25384,7 @@
         <v>0</v>
       </c>
       <c r="I167" s="2">
-        <v>8.5</v>
+        <v>10</v>
       </c>
       <c r="J167">
         <v>0</v>
@@ -25416,7 +25416,7 @@
         <v>10.3</v>
       </c>
       <c r="I168" s="2">
-        <v>7.9</v>
+        <v>9.5</v>
       </c>
       <c r="J168">
         <v>0</v>
@@ -25451,7 +25451,7 @@
         <v>25.9</v>
       </c>
       <c r="I169" s="2">
-        <v>7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J169">
         <v>0</v>
@@ -25521,7 +25521,7 @@
         <v>33.3</v>
       </c>
       <c r="I171" s="2">
-        <v>6.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J171">
         <v>0</v>
@@ -25556,7 +25556,7 @@
         <v>20.6</v>
       </c>
       <c r="I172" s="2">
-        <v>7.6</v>
+        <v>9</v>
       </c>
       <c r="J172">
         <v>0</v>
@@ -25591,7 +25591,7 @@
         <v>7.5</v>
       </c>
       <c r="I173" s="2">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
       <c r="J173">
         <v>0</v>
@@ -25626,7 +25626,7 @@
         <v>17.9</v>
       </c>
       <c r="I174" s="2">
-        <v>7.5</v>
+        <v>9.1</v>
       </c>
       <c r="J174">
         <v>0</v>
@@ -25661,7 +25661,7 @@
         <v>30</v>
       </c>
       <c r="I175" s="2">
-        <v>6.6</v>
+        <v>8.5</v>
       </c>
       <c r="J175">
         <v>0</v>
@@ -25696,7 +25696,7 @@
         <v>0</v>
       </c>
       <c r="I176" s="2">
-        <v>8.5</v>
+        <v>10</v>
       </c>
       <c r="J176">
         <v>0</v>
@@ -25731,7 +25731,7 @@
         <v>20.9</v>
       </c>
       <c r="I177" s="2">
-        <v>7.6</v>
+        <v>9</v>
       </c>
       <c r="J177">
         <v>0</v>
@@ -25763,7 +25763,7 @@
         <v>17.6</v>
       </c>
       <c r="I178" s="2">
-        <v>7.6</v>
+        <v>9.1</v>
       </c>
       <c r="J178">
         <v>0</v>
@@ -25798,7 +25798,7 @@
         <v>16.7</v>
       </c>
       <c r="I179" s="2">
-        <v>6.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J179">
         <v>0</v>
@@ -25833,7 +25833,7 @@
         <v>5.1</v>
       </c>
       <c r="I180" s="2">
-        <v>7.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J180">
         <v>0</v>
@@ -25868,7 +25868,7 @@
         <v>15.4</v>
       </c>
       <c r="I181" s="2">
-        <v>6.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J181">
         <v>0</v>
@@ -25938,7 +25938,7 @@
         <v>27</v>
       </c>
       <c r="I183" s="2">
-        <v>6.6</v>
+        <v>8.6</v>
       </c>
       <c r="J183">
         <v>0</v>
@@ -25973,7 +25973,7 @@
         <v>21.1</v>
       </c>
       <c r="I184" s="2">
-        <v>7.3</v>
+        <v>8.9</v>
       </c>
       <c r="J184">
         <v>0</v>
@@ -26008,7 +26008,7 @@
         <v>0</v>
       </c>
       <c r="I185" s="2">
-        <v>9.4</v>
+        <v>10</v>
       </c>
       <c r="J185">
         <v>0</v>
@@ -26043,7 +26043,7 @@
         <v>0</v>
       </c>
       <c r="I186" s="2">
-        <v>9.4</v>
+        <v>10</v>
       </c>
       <c r="J186">
         <v>0</v>
@@ -26075,7 +26075,7 @@
         <v>10.8</v>
       </c>
       <c r="I187" s="2">
-        <v>7.8</v>
+        <v>9.4</v>
       </c>
       <c r="J187">
         <v>0</v>
@@ -26110,7 +26110,7 @@
         <v>3.6</v>
       </c>
       <c r="I188" s="2">
-        <v>6.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J188">
         <v>0</v>
@@ -26145,7 +26145,7 @@
         <v>21.2</v>
       </c>
       <c r="I189" s="2">
-        <v>7.3</v>
+        <v>8.9</v>
       </c>
       <c r="J189">
         <v>0</v>
@@ -26180,7 +26180,7 @@
         <v>3</v>
       </c>
       <c r="I190" s="2">
-        <v>6.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J190">
         <v>0</v>
@@ -26215,7 +26215,7 @@
         <v>3.8</v>
       </c>
       <c r="I191" s="2">
-        <v>7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J191">
         <v>0</v>
@@ -26250,7 +26250,7 @@
         <v>15.4</v>
       </c>
       <c r="I192" s="2">
-        <v>7.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J192">
         <v>0</v>
@@ -26282,7 +26282,7 @@
         <v>9</v>
       </c>
       <c r="I193" s="2">
-        <v>7</v>
+        <v>9.5</v>
       </c>
       <c r="J193">
         <v>0</v>
@@ -26317,7 +26317,7 @@
         <v>6.7</v>
       </c>
       <c r="I194" s="2">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J194">
         <v>0</v>
@@ -26352,7 +26352,7 @@
         <v>0</v>
       </c>
       <c r="I195" s="2">
-        <v>9.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="J195">
         <v>0</v>
@@ -26387,7 +26387,7 @@
         <v>4.8</v>
       </c>
       <c r="I196" s="2">
-        <v>8.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J196">
         <v>0</v>
@@ -26422,7 +26422,7 @@
         <v>12.5</v>
       </c>
       <c r="I197" s="2">
-        <v>7.7</v>
+        <v>9.4</v>
       </c>
       <c r="J197">
         <v>0</v>
@@ -26454,7 +26454,7 @@
         <v>5.5</v>
       </c>
       <c r="I198" s="2">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J198">
         <v>0</v>
@@ -26524,7 +26524,7 @@
         <v>9.800000000000001</v>
       </c>
       <c r="I200" s="2">
-        <v>7.2</v>
+        <v>9.5</v>
       </c>
       <c r="J200">
         <v>0</v>
@@ -26559,7 +26559,7 @@
         <v>0</v>
       </c>
       <c r="I201" s="2">
-        <v>7.6</v>
+        <v>10</v>
       </c>
       <c r="J201">
         <v>0</v>
@@ -26591,7 +26591,7 @@
         <v>3.6</v>
       </c>
       <c r="I202" s="2">
-        <v>8.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J202">
         <v>0</v>
@@ -26626,7 +26626,7 @@
         <v>5.6</v>
       </c>
       <c r="I203" s="2">
-        <v>7.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J203">
         <v>0</v>
@@ -26661,7 +26661,7 @@
         <v>0</v>
       </c>
       <c r="I204" s="2">
-        <v>7.9</v>
+        <v>10</v>
       </c>
       <c r="J204">
         <v>0</v>
@@ -26696,7 +26696,7 @@
         <v>3.3</v>
       </c>
       <c r="I205" s="2">
-        <v>7.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J205">
         <v>0</v>
@@ -26731,7 +26731,7 @@
         <v>4</v>
       </c>
       <c r="I206" s="2">
-        <v>8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J206">
         <v>0</v>
@@ -26763,7 +26763,7 @@
         <v>3.3</v>
       </c>
       <c r="I207" s="2">
-        <v>7.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J207">
         <v>0</v>
@@ -26798,7 +26798,7 @@
         <v>55.6</v>
       </c>
       <c r="I208" s="2">
-        <v>5.5</v>
+        <v>7.2</v>
       </c>
       <c r="J208">
         <v>0</v>
@@ -26833,7 +26833,7 @@
         <v>46.2</v>
       </c>
       <c r="I209" s="2">
-        <v>5.6</v>
+        <v>7.7</v>
       </c>
       <c r="J209">
         <v>0</v>
@@ -26903,7 +26903,7 @@
         <v>46.2</v>
       </c>
       <c r="I211" s="2">
-        <v>5.6</v>
+        <v>7.7</v>
       </c>
       <c r="J211">
         <v>0</v>
@@ -26938,7 +26938,7 @@
         <v>47.4</v>
       </c>
       <c r="I212" s="2">
-        <v>5.7</v>
+        <v>7.6</v>
       </c>
       <c r="J212">
         <v>0</v>
@@ -26970,7 +26970,7 @@
         <v>59.3</v>
       </c>
       <c r="I213" s="2">
-        <v>5.5</v>
+        <v>7.1</v>
       </c>
       <c r="J213">
         <v>0</v>
@@ -27005,7 +27005,7 @@
         <v>5.9</v>
       </c>
       <c r="I214" s="2">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J214">
         <v>0</v>
@@ -27040,7 +27040,7 @@
         <v>2.5</v>
       </c>
       <c r="I215" s="2">
-        <v>8.300000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="J215">
         <v>0</v>
@@ -27075,7 +27075,7 @@
         <v>5.1</v>
       </c>
       <c r="I216" s="2">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J216">
         <v>0</v>
@@ -27110,7 +27110,7 @@
         <v>3.3</v>
       </c>
       <c r="I217" s="2">
-        <v>7.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J217">
         <v>0</v>
@@ -27180,7 +27180,7 @@
         <v>4</v>
       </c>
       <c r="I219" s="2">
-        <v>8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J219">
         <v>0</v>
@@ -27212,7 +27212,7 @@
         <v>4</v>
       </c>
       <c r="I220" s="2">
-        <v>8.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J220">
         <v>0</v>
@@ -27247,7 +27247,7 @@
         <v>7.5</v>
       </c>
       <c r="I221" s="2">
-        <v>7.7</v>
+        <v>9.6</v>
       </c>
       <c r="J221">
         <v>0</v>
@@ -27279,7 +27279,7 @@
         <v>7.5</v>
       </c>
       <c r="I222" s="2">
-        <v>7.7</v>
+        <v>9.6</v>
       </c>
       <c r="J222">
         <v>0</v>
@@ -27314,7 +27314,7 @@
         <v>27.8</v>
       </c>
       <c r="I223" s="2">
-        <v>7.1</v>
+        <v>8.6</v>
       </c>
       <c r="J223">
         <v>0</v>
@@ -27346,7 +27346,7 @@
         <v>27.8</v>
       </c>
       <c r="I224" s="2">
-        <v>7.1</v>
+        <v>8.6</v>
       </c>
       <c r="J224">
         <v>0</v>
@@ -27381,7 +27381,7 @@
         <v>3.8</v>
       </c>
       <c r="I225" s="2">
-        <v>8.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J225">
         <v>0</v>
@@ -27413,7 +27413,7 @@
         <v>3.8</v>
       </c>
       <c r="I226" s="2">
-        <v>8.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J226">
         <v>0</v>
@@ -27448,7 +27448,7 @@
         <v>66.7</v>
       </c>
       <c r="I227" s="2">
-        <v>5.6</v>
+        <v>6.7</v>
       </c>
       <c r="J227">
         <v>0</v>
@@ -27483,7 +27483,7 @@
         <v>48.6</v>
       </c>
       <c r="I228" s="2">
-        <v>5.9</v>
+        <v>7.6</v>
       </c>
       <c r="J228">
         <v>0</v>
@@ -27518,7 +27518,7 @@
         <v>31.6</v>
       </c>
       <c r="I229" s="2">
-        <v>6.1</v>
+        <v>8.4</v>
       </c>
       <c r="J229">
         <v>0</v>
@@ -27553,7 +27553,7 @@
         <v>14.3</v>
       </c>
       <c r="I230" s="2">
-        <v>7.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J230">
         <v>0</v>
@@ -27588,7 +27588,7 @@
         <v>7.1</v>
       </c>
       <c r="I231" s="2">
-        <v>7.9</v>
+        <v>9.6</v>
       </c>
       <c r="J231">
         <v>0</v>
@@ -27623,7 +27623,7 @@
         <v>7.1</v>
       </c>
       <c r="I232" s="2">
-        <v>7.9</v>
+        <v>9.6</v>
       </c>
       <c r="J232">
         <v>0</v>
@@ -27655,7 +27655,7 @@
         <v>31.8</v>
       </c>
       <c r="I233" s="2">
-        <v>6.8</v>
+        <v>8.5</v>
       </c>
       <c r="J233">
         <v>0</v>
@@ -27690,7 +27690,7 @@
         <v>12</v>
       </c>
       <c r="I234" s="2">
-        <v>8.4</v>
+        <v>9.4</v>
       </c>
       <c r="J234">
         <v>0</v>
@@ -27725,7 +27725,7 @@
         <v>11.8</v>
       </c>
       <c r="I235" s="2">
-        <v>8.4</v>
+        <v>9.4</v>
       </c>
       <c r="J235">
         <v>0</v>
@@ -27757,7 +27757,7 @@
         <v>11.9</v>
       </c>
       <c r="I236" s="2">
-        <v>8.4</v>
+        <v>9.4</v>
       </c>
       <c r="J236">
         <v>0</v>
@@ -27792,7 +27792,7 @@
         <v>0</v>
       </c>
       <c r="I237" s="2">
-        <v>8.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="J237">
         <v>0</v>
@@ -27827,7 +27827,7 @@
         <v>0</v>
       </c>
       <c r="I238" s="2">
-        <v>8.699999999999999</v>
+        <v>10</v>
       </c>
       <c r="J238">
         <v>0</v>
@@ -27859,7 +27859,7 @@
         <v>0</v>
       </c>
       <c r="I239" s="2">
-        <v>8.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="J239">
         <v>0</v>
@@ -27894,7 +27894,7 @@
         <v>15.4</v>
       </c>
       <c r="I240" s="2">
-        <v>7.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J240">
         <v>0</v>
@@ -27926,7 +27926,7 @@
         <v>15.4</v>
       </c>
       <c r="I241" s="2">
-        <v>7.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J241">
         <v>0</v>
@@ -27996,7 +27996,7 @@
         <v>17.9</v>
       </c>
       <c r="I243" s="2">
-        <v>6.9</v>
+        <v>9.1</v>
       </c>
       <c r="J243">
         <v>0</v>
@@ -28031,7 +28031,7 @@
         <v>21.6</v>
       </c>
       <c r="I244" s="2">
-        <v>7</v>
+        <v>8.9</v>
       </c>
       <c r="J244">
         <v>0</v>
@@ -28066,7 +28066,7 @@
         <v>15.8</v>
       </c>
       <c r="I245" s="2">
-        <v>7.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J245">
         <v>0</v>
@@ -28101,7 +28101,7 @@
         <v>3.8</v>
       </c>
       <c r="I246" s="2">
-        <v>8.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J246">
         <v>0</v>
@@ -28133,7 +28133,7 @@
         <v>13.8</v>
       </c>
       <c r="I247" s="2">
-        <v>7.9</v>
+        <v>9.4</v>
       </c>
       <c r="J247">
         <v>0</v>
@@ -28168,7 +28168,7 @@
         <v>14.8</v>
       </c>
       <c r="I248" s="2">
-        <v>7.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J248">
         <v>0</v>
@@ -28203,7 +28203,7 @@
         <v>16.7</v>
       </c>
       <c r="I249" s="2">
-        <v>7.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J249">
         <v>0</v>
@@ -28238,7 +28238,7 @@
         <v>7.7</v>
       </c>
       <c r="I250" s="2">
-        <v>8</v>
+        <v>9.6</v>
       </c>
       <c r="J250">
         <v>0</v>
@@ -28273,7 +28273,7 @@
         <v>3.3</v>
       </c>
       <c r="I251" s="2">
-        <v>7.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J251">
         <v>0</v>
@@ -28308,7 +28308,7 @@
         <v>4</v>
       </c>
       <c r="I252" s="2">
-        <v>8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J252">
         <v>0</v>
@@ -28343,7 +28343,7 @@
         <v>0</v>
       </c>
       <c r="I253" s="2">
-        <v>7.9</v>
+        <v>10</v>
       </c>
       <c r="J253">
         <v>0</v>
@@ -28375,7 +28375,7 @@
         <v>7.2</v>
       </c>
       <c r="I254" s="2">
-        <v>7.7</v>
+        <v>9.6</v>
       </c>
       <c r="J254">
         <v>0</v>
@@ -28410,7 +28410,7 @@
         <v>12.8</v>
       </c>
       <c r="I255" s="2">
-        <v>6.9</v>
+        <v>9.4</v>
       </c>
       <c r="J255">
         <v>0</v>
@@ -28445,7 +28445,7 @@
         <v>20.5</v>
       </c>
       <c r="I256" s="2">
-        <v>6.2</v>
+        <v>9</v>
       </c>
       <c r="J256">
         <v>0</v>
@@ -28480,7 +28480,7 @@
         <v>16.2</v>
       </c>
       <c r="I257" s="2">
-        <v>6.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J257">
         <v>0</v>
@@ -28515,7 +28515,7 @@
         <v>15.8</v>
       </c>
       <c r="I258" s="2">
-        <v>6.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J258">
         <v>0</v>
@@ -28550,7 +28550,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="I259" s="2">
-        <v>7.2</v>
+        <v>9.6</v>
       </c>
       <c r="J259">
         <v>0</v>
@@ -28585,7 +28585,7 @@
         <v>0</v>
       </c>
       <c r="I260" s="2">
-        <v>7.8</v>
+        <v>10</v>
       </c>
       <c r="J260">
         <v>0</v>
@@ -28617,7 +28617,7 @@
         <v>12.8</v>
       </c>
       <c r="I261" s="2">
-        <v>6.9</v>
+        <v>9.4</v>
       </c>
       <c r="J261">
         <v>0</v>
@@ -28652,7 +28652,7 @@
         <v>30.6</v>
       </c>
       <c r="I262" s="2">
-        <v>6.8</v>
+        <v>8.5</v>
       </c>
       <c r="J262">
         <v>0</v>
@@ -28687,7 +28687,7 @@
         <v>0</v>
       </c>
       <c r="I263" s="2">
-        <v>8.1</v>
+        <v>10</v>
       </c>
       <c r="J263">
         <v>0</v>
@@ -28722,7 +28722,7 @@
         <v>0</v>
       </c>
       <c r="I264" s="2">
-        <v>7.6</v>
+        <v>10</v>
       </c>
       <c r="J264">
         <v>0</v>
@@ -28757,7 +28757,7 @@
         <v>0</v>
       </c>
       <c r="I265" s="2">
-        <v>8.5</v>
+        <v>10</v>
       </c>
       <c r="J265">
         <v>0</v>
@@ -28792,7 +28792,7 @@
         <v>0</v>
       </c>
       <c r="I266" s="2">
-        <v>8.5</v>
+        <v>10</v>
       </c>
       <c r="J266">
         <v>0</v>
@@ -28824,7 +28824,7 @@
         <v>7.6</v>
       </c>
       <c r="I267" s="2">
-        <v>7.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J267">
         <v>0</v>
@@ -28859,7 +28859,7 @@
         <v>0</v>
       </c>
       <c r="I268" s="2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J268">
         <v>0</v>
@@ -28894,7 +28894,7 @@
         <v>0</v>
       </c>
       <c r="I269" s="2">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="J269">
         <v>0</v>
@@ -28929,7 +28929,7 @@
         <v>0</v>
       </c>
       <c r="I270" s="2">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="J270">
         <v>0</v>
@@ -28964,7 +28964,7 @@
         <v>0</v>
       </c>
       <c r="I271" s="2">
-        <v>9.4</v>
+        <v>10</v>
       </c>
       <c r="J271">
         <v>0</v>
@@ -28999,7 +28999,7 @@
         <v>0</v>
       </c>
       <c r="I272" s="2">
-        <v>9.4</v>
+        <v>10</v>
       </c>
       <c r="J272">
         <v>0</v>
@@ -29031,7 +29031,7 @@
         <v>0</v>
       </c>
       <c r="I273" s="2">
-        <v>9.4</v>
+        <v>10</v>
       </c>
       <c r="J273">
         <v>0</v>

</xml_diff>